<commit_message>
watchlist: Vylor rehecha (ratings y FCF@5y propios; múltiplos de Roger sin cambio)
- Ratings de la fila 73 rehechos para el negocio de semillas solo (New Corteva se lleva la
  protección de cultivos, los genéricos, el acuerdo con la FTC y los pasivos de DuPont):
  R1 4,38 -> 5,63, R2 5,90 -> 6,40, R3 6,43 -> 6,57; compuesto 5,81 -> 6,31. Detalle en la
  hoja Updates Log (fila 261).
- FCF@5y 2.046 / 3.295 -> 2.200 / 3.320, sobre un FCF limpio de partida de ~1.900 (FY25 2.118
  y LTM sin el pago único a Bayer, menos los intereses de la deuda de la escisión).
- Múltiplos 14x / 22x sin cambio, por decisión de Roger. TIR -10,1% / +9,0% a 67,26 $; el
  bajista pierde un 41% (cumple el test del 15%).
- tools/build_pack.py: veredicto de Vylor (3,5/5, 0-1%, ampliar bajo 51 $).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/watchlist_ratings.xlsx
+++ b/data/raw/watchlist_ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roger\Cosas Roger\BOLSA E INVERSIÓN\repos\watchlist-dashboard\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5760E5-D41A-4378-BB35-722FED9AF3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F921A8-4BF1-4221-B18E-1896E0DA6004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2664,7 +2664,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1975" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1979" uniqueCount="918">
   <si>
     <t>WATCHLIST RATINGS — JP Morgan Equity Research Framework | Long-Term Investor View</t>
   </si>
@@ -5439,10 +5439,22 @@
     <t>FUENTE: notas de resultados FY25 (24-feb-2026) y H1-26 (28-jul-2026) e informe financiero semestral 2026 de Verallia. LTM = FY25 + H1-26 - H1-25. Ingresos 3.331,5 + 1.698,8 - 1.722,6 = 3.307,7; EBITDA ajustado LTM 693,0 (de la compania). FCF de Verallia (EBITDA aj. - capex +/- circulante - otros impactos operativos, que incluyen el efecto de caja de la NIIF 16 - intereses - impuestos): 166,0 + 102,0 - 66,2 = 201,8, menos SBC 6,2 (estado de cambios en el patrimonio) = 195,6 (incluye 19 de reestructuracion en el H1-26). La fila llevaba 249 (sin fuente). Caja 413,9; deuda bruta 2.192,8 - arrendamientos 60,9 = 2.131,9 (deuda neta de la compania 1.778,9). Capex 246 &lt; amortizacion: sin normalizar. NOPAT pendiente. Q3: 27-oct-2026 (calendario de la compania)</t>
   </si>
   <si>
-    <t>VYLOR (semillas de Corteva) desde el 1-oct-2026, sustituye a CTVA por decision de Roger (2-oct). FUENTE: Form 10 de Vylor (EDGAR, 21-sep-2026): estados combinados del negocio de semillas. LTM = FY25 + H1-26 - H1-25. Ventas 9.898 + 7.555 - 7.244 = 10.209. EBITDA operativo del segmento 2.636 + 3.000 - 2.705 = 2.931 (antes de costes corporativos; pro forma FY25 2.503). Flujo de explotacion 2.506 - 2.471 + 1.557 = 1.592 - capex 350 - SBC 47 = 1.195: INCLUYE el pago unico a Bayer por el litigio (cargo de 610 en FY25, pagado en el H1-26); sin el ~1.800; FY25 2.118. Capex de crecimiento 350 - depreciacion 317 = 33 -&gt; BS 1.228. NOPAT ~1.172 (EBIT FY25 sin Bayer 1.562 x 75%). Caja 1.100 y deuda 5.659 pro forma a 30-jun-2026; capital empleado = fondos propios pro forma 12.268 + deuda neta. FCF@5y, multiplos y ratings son los de la Corteva combinada: PENDIENTES DE ROGER. Q3: ~5-nov-2026 (estimado)</t>
-  </si>
-  <si>
     <t>FUENTE: 10-K FY26 (EDGAR XBRL) + 8-K Q1 FY27 (1-oct-2026). Ingresos LTM = 46.398 + 11.213 - 11.720 = 45.891. FCF - SBC FY26 = OCF 2.868 - capex 684 - SBC 715 = 1.469 (el 10-Q del Q1 aun no esta: LTM de caja pendiente). Caja 6.903 + 1.465 = 8.368; deuda financiera 2.000 + 5.893 = 7.893 (sin arrendamientos operativos; la fila llevaba 11.040). EBITDA y NOPAT pendientes del 10-Q. Guia FY27: ventas -HSD, BPA aj. 1,15-1,35; plan Pace (1.000 M$ de cargos, 2.500 de ahorro hasta FY31). Investor Day en noviembre. Proximos: ~18-dic-2026 (estimado) | 2-oct: FCF@5y 2.823 / 6.005 (escenarios 'marca madura estancada' y 'recuperacion completa' del deep dive NKE_Deep_Dive.md), por decision de Roger; multiplos 14x / 21x sin cambio</t>
+  </si>
+  <si>
+    <t>VYLOR (semillas de Corteva) desde el 1-oct-2026, sustituye a CTVA por decision de Roger (2-oct). FUENTE: Form 10 de Vylor (EDGAR, 21-sep-2026): estados combinados del negocio de semillas. LTM = FY25 + H1-26 - H1-25. Ventas 9.898 + 7.555 - 7.244 = 10.209. EBITDA operativo del segmento 2.636 + 3.000 - 2.705 = 2.931 (antes de costes corporativos; pro forma FY25 2.503). Flujo de explotacion 2.506 - 2.471 + 1.557 = 1.592 - capex 350 - SBC 47 = 1.195: INCLUYE el pago unico a Bayer por el litigio (cargo de 610 en FY25, pagado en el H1-26); sin el ~1.800; FY25 2.118. Capex de crecimiento 350 - depreciacion 317 = 33 -&gt; BS 1.228. NOPAT ~1.172 (EBIT FY25 sin Bayer 1.562 x 75%). Caja 1.100 y deuda 5.659 pro forma a 30-jun-2026; capital empleado = fondos propios pro forma 12.268 + deuda neta. | 2-oct (Roger: 'rehaz todo con Vylor, sin tocar los multiplos'): FCF@5y 2.200 / 3.320 sobre un FCF limpio de partida ~1.900 (FY25 2.118 y LTM sin Bayer ~1.800, menos ~130 de intereses netos de la deuda de la escision: cargo pro forma 170). Bajista: ventas +2%/anio, margen FCF 19,5% -&gt; 2.200 (+3%/anio). Alcista: ventas +5%/anio (precio +3% como en 2024-26, licencias), margen 25,5% por el giro de regalias (coste neto 439 en 2025 -&gt; neutral en 2026 -&gt; +1.000 en 2035) -&gt; 3.320 (+12%/anio). OJO: el crecimiento implicito de BE/BG se calcula contra AS (1.195, deprimido por Bayer) y sale inflado; contra 1.900 es +3% / +12%. Multiplos 14x / 22x de Roger SIN CAMBIO. Ratings rehechos para semillas: ver Updates Log del 2-oct. Q3: ~5-nov-2026 (estimado)</t>
+  </si>
+  <si>
+    <t>VYLR</t>
+  </si>
+  <si>
+    <t>ALTA por sustitucion de CTVA. A (tipo de dato), AP-AV, AZ, BQ-BT, ratings R1/R2/R3, BD/BF</t>
+  </si>
+  <si>
+    <t>Form 10 de Vylor (EDGAR, 21-sep-2026) y 8-K de Corteva del 1-oct-2026</t>
+  </si>
+  <si>
+    <t>Vylor sustituye a Corteva (escision del 1-oct-2026; la semilla, con el foso de la tesis, es Vylor). Roger: 'rehaz todo con Vylor, sin tocar los multiplos'. RATINGS (solo lo que cambia con la escision; New Corteva se lleva la proteccion de cultivos, los genericos, el acuerdo con la FTC y los pasivos heredados de DuPont): R1 MOAT 6-&gt;7 (recompra anual obligada de semilla hibrida, Pioneer n1 en maiz y soja de EE.UU., Enlist E3 en ~65% de la soja de EE.UU.), Optionality 1-&gt;2 (2a cartera de patentes de edicion genetica, trigo hibrido en 2027, licencias hacia +1.000 M$ netos en 2035). R2 Financials 11-&gt;12 (EBITDA de segmento 26,6% y +340 pb en 2025; FCF ~19% de ventas frente a 3% de proteccion de cultivos), MOAT 15-&gt;16, Potential 11-&gt;12, Risks -11-&gt;-9 (sin genericos, FTC ni pasivos de DuPont; quedan aprobaciones regulatorias, clima, Brasil y la deuda nueva). R3 Financing -&gt; 3-&gt;2 (5.659 M$ de deuda nueva por la escision, 3.499 pagados a New Corteva), MOAT Structural 12-&gt;13, Terminal Risk -4-&gt;-3. Resto sin cambio. Compuesto 5,81 -&gt; 6,31. FCF@5y 2.046/3.295 -&gt; 2.200/3.320 sobre un FCF limpio de ~1.900 (+3% / +12% anual). Multiplos 14x / 22x SIN CAMBIO. Test del bajista: valor 39,3 $ frente a 67,26 $, -41% (cumple el minimo del 15%). Multiplos dentro del anclaje 0,75x / 1,25x del EV/FCF limpio de hoy (~26x).</t>
   </si>
 </sst>
 </file>
@@ -6380,7 +6392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="183">
+  <cellXfs count="184">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6846,6 +6858,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7659,7 +7672,7 @@
                   <c:v>-0.18948800194233184</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.8334361539594806E-2</c:v>
+                  <c:v>4.8381582213031127E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>5.9461744408414008E-2</c:v>
@@ -9727,15 +9740,15 @@
     <v>283.10000000000002</v>
     <v>0.91410000000000002</v>
     <v>-8.7100000000000009</v>
-    <v>6.2199999999999994E-4</v>
+    <v>2.0011999999999999E-2</v>
     <v>-3.0893999999999998E-2</v>
-    <v>0.17</v>
+    <v>5.47</v>
     <v>44236722336</v>
     <v>281.93</v>
     <v>Veeva Systems Inc. Es un proveedor de soluciones en la nube para la industria global de las ciencias de la vida. Ofrece software SPAN Cloud, datos y consultoría empresarial, y está diseñado para satisfacer las necesidades de sus clientes y las funciones estratégicas de negocio, desde la investigación y el desarrollo (I+D) hasta la comercialización. Sus cuatro categorías de productos incluyen Veeva Development Cloud, Veeva Quality Cloud, Veeva Commercial Cloud y Veeva Data Cloud. Veeva Development Cloud incluye paquetes de aplicaciones para las funciones clínicas, regulatorias y de seguridad de las empresas de ciencias de la vida, todo construido en su plataforma Veeva Vault. Veeva Quality Cloud unifica aplicaciones, procesos y socios en las soluciones de gestión de contenido, capacitación, gestión de calidad, garantía y laboratorio de control en la plataforma Veeva Vault. Veeva Commercial Cloud es una categoría de producto compuesta por soluciones de software y análisis. Veeva Data Cloud es una plataforma de datos compuesta por datos de referencia conectados, datos profundos y datos de transacciones.</v>
     <v>7928</v>
     <v>XNYS</v>
-    <v>46297.853689860938</v>
+    <v>46297.869885914064</v>
     <v>New York Stock Exchange</v>
     <v>0</v>
     <v>284.58999999999997</v>
@@ -9747,13 +9760,13 @@
     <v>VEEVA SYSTEMS INC.</v>
     <v>44.682499999999997</v>
     <v>273.22000000000003</v>
-    <v>273.5</v>
+    <v>278.8</v>
     <v>Healthcare Equipment &amp; Supplies</v>
     <v>4280 Hacienda Drive, PLEASANTON, CA, 94588 US</v>
     <v>VEEV</v>
     <v>Acciones</v>
     <v>VEEVA SYSTEMS INC. (XNYS:VEEV)</v>
-    <v>1077576</v>
+    <v>1077697</v>
     <v>1849777</v>
   </rv>
   <rv s="2">
@@ -9810,7 +9823,7 @@
     <v>Microsoft Corporation es una empresa de tecnología. La Compañía desarrolla y apoya software, servicios, dispositivos y soluciones. Los segmentos de la compañía incluyen Productividad y Procesos de Negocio, Nube Inteligente y más Informática Personal. El segmento Productividad y Procesos de Negocio está formado por productos y servicios en su cartera de servicios de productividad, comunicación e información. Este segmento comprende principalmente: Office Commercial, Office Consumer, LinkedIn y soluciones empresariales de Dynamics. El segmento de la nube inteligente consiste en productos de servidor y servicios en la nube, incluidos Azure y otros servicios en la nube, SQL Server, Windows Server, Visual Studio, System Center y Windows Server. licencias de acceso de clientes (CAL) relacionadas, Nuance y GitHub; y Servicios empresariales, incluidos los servicios de soporte empresarial, las soluciones de la industria y los servicios profesionales de Nuance. El segmento más personal de Computación comprende principalmente Windows, dispositivos, juegos y publicidad de búsqueda y noticias.</v>
     <v>223000</v>
     <v>XNAS</v>
-    <v>46297.855688529686</v>
+    <v>46297.87231398125</v>
     <v>6</v>
     <v>Nasdaq Stock Market</v>
     <v>7</v>
@@ -9829,7 +9842,7 @@
     <v>MSFT</v>
     <v>Acciones</v>
     <v>MICROSOFT CORPORATION (XNAS:MSFT)</v>
-    <v>17147700</v>
+    <v>17178193</v>
     <v>22115939</v>
   </rv>
   <rv s="2">
@@ -9910,15 +9923,15 @@
     <v>37.14</v>
     <v>1.56</v>
     <v>0.38500000000000001</v>
-    <v>7.3129999999999992E-3</v>
+    <v>7.5839999999999996E-3</v>
     <v>1.0536E-2</v>
-    <v>0.27</v>
+    <v>0.28000000000000003</v>
     <v>90540506175</v>
     <v>36.54</v>
     <v>Brookfield Corporation es una firma de inversión global con sede en Canadá enfocada en la construcción de riqueza a largo plazo para instituciones e individuos de todo el mundo. La Compañía tiene tres negocios principales: Gestión de activos alternativos, Soluciones de patrimonio y sus negocios operativos, que se encuentran en energía renovable, infraestructura, servicios empresariales e industriales, y bienes raíces. Su negocio de gestión de activos incluye la gestión de fondos privados a largo plazo, estrategias perpetuas y estrategias líquidas en nombre de sus inversores y de sí mismo. El negocio de Wealth Solutions de la Compañía incluye su participación contabilizada en Brookfield Wealth Solutions Ltd. Su negocio de energía renovable y transición incluye la propiedad, operación y desarrollo de activos de generación de energía solar hidroeléctrica, eólica, a escala de servicios públicos, energía distribuida y soluciones sostenibles. El negocio de infraestructura de la Compañía incluye la propiedad, operación y desarrollo de servicios públicos, transporte, midstream y activos de datos.</v>
     <v>250000</v>
     <v>XNYS</v>
-    <v>46297.853615520311</v>
+    <v>46297.870753969532</v>
     <v>New York Stock Exchange</v>
     <v>13</v>
     <v>37.270000000000003</v>
@@ -9930,13 +9943,13 @@
     <v>Brookfield Corporation</v>
     <v>72.203800000000001</v>
     <v>36.924999999999997</v>
-    <v>37.19</v>
+    <v>37.200000000000003</v>
     <v>Investment Banking &amp; Investment Services</v>
     <v>Brookfield Place, 181 Bay St, Ste 100, Po Box 762, TORONTO, ON, M5J 2T3 CA</v>
     <v>BN</v>
     <v>Acciones</v>
     <v>Brookfield Corporation (XNYS:BN)</v>
-    <v>6441320</v>
+    <v>6441352</v>
     <v>4949765</v>
   </rv>
   <rv s="2">
@@ -9965,15 +9978,15 @@
     <v>921.18</v>
     <v>0.86319999999999997</v>
     <v>5.71</v>
-    <v>-1.0460000000000001E-3</v>
+    <v>-2.6829999999999996E-3</v>
     <v>6.241E-3</v>
-    <v>-0.96340000000000003</v>
+    <v>-2.4700000000000002</v>
     <v>408092842900</v>
     <v>914.94</v>
     <v>Costco Wholesale Corporation (Costco) opera almacenes de membresía y sitios de comercio electrónico que ofrecen una selección de productos de marca nacional y de marca privada en una amplia gama de categorías. La Compañía compra la mayoría de sus mercancías directamente a los proveedores y la dirige a puntos de consolidación de cross-docking (depósitos) o directamente a sus almacenes. Opera 891 almacenes, incluyendo 614 en los Estados Unidos y Puerto Rico, 108 en Canadá, 40 en México, 35 en Japón, 29 en el Reino Unido, 19 en Corea, 15 en Australia, 14 en Taiwán, siete en China, y más. cinco en España, dos en Francia, y uno en Islandia, Nueva Zelanda y Suecia. También opera sitios de comercio electrónico en los Estados Unidos, Canadá, el Reino Unido, México, Corea, Taiwán, Japón y Australia. La Compañía ofrece una amplia selección de mercancías, además de la conveniencia de departamentos especializados y servicios exclusivos para miembros.</v>
     <v>341000</v>
     <v>XNAS</v>
-    <v>46297.855544941405</v>
+    <v>46297.872210890622</v>
     <v>Nasdaq Stock Market</v>
     <v>16</v>
     <v>921.18</v>
@@ -9985,13 +9998,13 @@
     <v>COSTCO WHOLESALE CORPORATION</v>
     <v>44.348799999999997</v>
     <v>920.65</v>
-    <v>919.6866</v>
+    <v>918.18</v>
     <v>Diversified Retail</v>
     <v>999 Lake Dr, ISSAQUAH, WA, 98027- US</v>
     <v>COST</v>
     <v>Acciones</v>
     <v>COSTCO WHOLESALE CORPORATION (XNAS:COST)</v>
-    <v>2011443</v>
+    <v>2011680</v>
     <v>2318063</v>
   </rv>
   <rv s="2">
@@ -10127,15 +10140,15 @@
     <v>201.18</v>
     <v>0.85629999999999995</v>
     <v>-2.1800000000000002</v>
-    <v>-2.2889999999999998E-3</v>
+    <v>1.0169999999999999E-3</v>
     <v>-1.0966999999999999E-2</v>
-    <v>-0.45</v>
+    <v>0.2</v>
     <v>32056554020</v>
     <v>198.78</v>
     <v>Zscaler, Inc. Es una compañía de seguridad en la nube. La Compañía ha desarrollado una plataforma que incorpora funcionalidades de seguridad básicas necesarias para permitir un acceso rápido y seguro a los recursos de la nube basado en la identidad, el contexto y las políticas de una organización. Su plataforma Zscaler Zero Trust Exchange protege a miles de clientes de ciberataques y pérdida de datos conectando de forma segura a usuarios, dispositivos y aplicaciones en cualquier ubicación. Su solución es una plataforma en la nube distribuida, multiusuario y diseñada específicamente que incorpora la funcionalidad de seguridad necesaria para permitir que los usuarios, aplicaciones y dispositivos utilicen de manera segura y eficiente aplicaciones y servicios autorizados basados en las políticas de negocio de una organización. Ofrece sus soluciones utilizando un modelo de negocio de software como servicio (SaaS) y vende suscripciones a los clientes para acceder a su plataforma en la nube, junto con los servicios de soporte relacionados. Ofrece una plataforma de seguridad que combina su plataforma con operaciones de seguridad automatizadas.</v>
     <v>8700</v>
     <v>XNAS</v>
-    <v>46297.85512490703</v>
+    <v>46297.869378078125</v>
     <v>Nasdaq Stock Market</v>
     <v>25</v>
     <v>202</v>
@@ -10147,13 +10160,13 @@
     <v>ZSCALER, INC.</v>
     <v>0</v>
     <v>196.6</v>
-    <v>196.15</v>
+    <v>196.8</v>
     <v>Software &amp; IT Services</v>
     <v>120 Holger Way, SAN JOSE, CA, 95134 US</v>
     <v>ZS</v>
     <v>Acciones</v>
     <v>ZSCALER, INC. (XNAS:ZS)</v>
-    <v>1719210</v>
+    <v>1720615</v>
     <v>3644664</v>
   </rv>
   <rv s="2">
@@ -10234,15 +10247,15 @@
     <v>251.505</v>
     <v>1.492</v>
     <v>3.29</v>
-    <v>-5.1690000000000004E-4</v>
+    <v>-3.0430000000000001E-3</v>
     <v>1.3253999999999998E-2</v>
-    <v>-0.13</v>
+    <v>-0.76529999999999998</v>
     <v>2712972691200</v>
     <v>248.23</v>
     <v>Amazon.com, Inc. Ofrece una gama de productos y servicios a los clientes. Los productos ofrecidos a través de sus tiendas incluyen mercancía y contenido que ha adquirido para su reventa y productos ofrecidos por terceros vendedores. Los segmentos de la compañía incluyen Norteamérica, International y Amazon Web Services (AWS). Sirve a los consumidores a través de sus tiendas en línea y físicas y se centra en la selección, el precio y la conveniencia. Los clientes acceden a sus ofertas a través de sus sitios web, aplicaciones móviles, Alexa, dispositivos, streaming, y visitando físicamente sus tiendas. También fabrica y vende dispositivos electrónicos, incluyendo Kindle, tableta de fuego, Fire TV, Echo, Ring, Blink y eero, y desarrolla y produce contenido multimedia. Presta servicios a desarrolladores y empresas de todos los tamaños, incluidas empresas emergentes, agencias gubernamentales e instituciones académicas, a través de AWS, que ofrece un conjunto de servicios de tecnología bajo demanda, incluyendo computación, almacenamiento, base de datos, análisis, y el aprendizaje automático, y otros servicios.</v>
     <v>1595000</v>
     <v>XNAS</v>
-    <v>46297.855744745313</v>
+    <v>46297.872399478903</v>
     <v>Nasdaq Stock Market</v>
     <v>31</v>
     <v>253.55770000000001</v>
@@ -10252,15 +10265,15 @@
     <v>USD</v>
     <v>AMAZON.COM, INC.</v>
     <v>AMAZON.COM, INC.</v>
-    <v>20.230699999999999</v>
+    <v>19.966000000000001</v>
     <v>251.52</v>
-    <v>251.39</v>
+    <v>250.75470000000001</v>
     <v>Diversified Retail</v>
     <v>410 Terry Avenue North, SEATTLE, WA, 98109 US</v>
     <v>AMZN</v>
     <v>Acciones</v>
     <v>AMAZON.COM, INC. (XNAS:AMZN)</v>
-    <v>33018438</v>
+    <v>33045393</v>
     <v>35374853</v>
   </rv>
   <rv s="2">
@@ -10497,15 +10510,15 @@
     <v>614</v>
     <v>1.3813</v>
     <v>-0.32</v>
-    <v>7.561E-4</v>
+    <v>2.6770000000000001E-3</v>
     <v>-4.8359999999999999E-4</v>
-    <v>0.5</v>
+    <v>1.77</v>
     <v>14285327025</v>
     <v>661.75</v>
     <v>Fair Isaac Corporation es una empresa de software de análisis aplicado. La compañía se centra en el uso de análisis predictivos y ciencia de datos para mejorar las decisiones operativas. La Compañía opera a través de dos segmentos: Puntajes y Software. El segmento de puntajes incluye las soluciones y servicios de puntaje de negocios a negocios de la Compañía que dan a sus clientes acceso a crédito predictivo y otros puntajes. Este segmento incluye sus soluciones de puntuación entre empresas y consumidores, incluidas sus ofertas de suscripción de myFICO.com. El segmento de software de la compañía incluye soluciones de análisis y gestión de decisiones preconfiguradas diseñadas para un tipo específico de necesidad o proceso de negocio, como originación de cuentas, gestión de clientes, participación de clientes, detección de fraude y marketing, así como servicios profesionales asociados. Este segmento incluye FICO Platform, una oferta de software modular diseñada para soportar casos de uso analítico y de decisión avanzados, así como software analítico y de toma de decisiones independiente.</v>
     <v>3876</v>
     <v>XNYS</v>
-    <v>46297.855152707809</v>
+    <v>46297.872282858596</v>
     <v>New York Stock Exchange</v>
     <v>46</v>
     <v>675.5</v>
@@ -10517,13 +10530,13 @@
     <v>FAIR ISAAC CORPORATION</v>
     <v>19.108499999999999</v>
     <v>661.43</v>
-    <v>661.75</v>
+    <v>663.02</v>
     <v>Software &amp; IT Services</v>
     <v>5 West Mendenhall, Suites 105, BOZEMAN, MT, 59715 US</v>
     <v>FICO</v>
     <v>Acciones</v>
     <v>FAIR ISAAC CORPORATION (XNYS:FICO)</v>
-    <v>1641440</v>
+    <v>1643094</v>
     <v>768832</v>
   </rv>
   <rv s="2">
@@ -10652,22 +10665,22 @@
     <v>3</v>
     <v>4</v>
     <v>Finance</v>
-    <v>5</v>
+    <v>17</v>
     <v>XNAS</v>
     <v>1956016000</v>
     <v>2014</v>
     <v>42.37</v>
     <v>0.53520000000000001</v>
     <v>0.8</v>
-    <v>0</v>
+    <v>9.525E-4</v>
     <v>1.8984000000000001E-2</v>
-    <v>0</v>
+    <v>4.0899999999999999E-2</v>
     <v>83991327040</v>
     <v>42.14</v>
     <v>Monster Beverage Corporation es una sociedad holding. La Compañía, a través de sus subsidiarias, desarrolla, comercializa, vende y distribuye bebidas de bebidas energéticas y concentrados para bebidas energéticas bajo diversas marcas. Su segmento de bebidas Monster Energy consiste principalmente en sus bebidas energéticas Monster Energy, bebidas energéticas de alto rendimiento Reign Total Body Fuel, bebidas energéticas de bienestar total Reign Storm y bebidas energéticas Bang Energy. Su segmento de Marcas Estratégicas consiste principalmente en varias marcas de bebidas energéticas adquiridas de The Coca-Cola Company, así como sus marcas de energía asequibles, Predator y Fury. Su segmento de marcas de alcohol consiste en varias cervezas artesanales, seltzers duros y bebidas de malta con sabor. Su otro segmento consiste en ciertos productos vendidos por American Fruits and Flavors LLC, una subsidiaria de propiedad total de la Compañía, a clientes independientes de terceros. También desarrolla, comercializa, vende y distribuye aguas tranquilas y chispeantes bajo la marca Monster Tour Water.</v>
     <v>6891</v>
     <v>XNAS</v>
-    <v>46297.847224930469</v>
+    <v>46297.860535995314</v>
     <v>Nasdaq Stock Market</v>
     <v>55</v>
     <v>42.984999999999999</v>
@@ -10679,13 +10692,13 @@
     <v>MONSTER BEVERAGE CORPORATION</v>
     <v>39.851500000000001</v>
     <v>42.94</v>
-    <v>42.94</v>
+    <v>42.980899999999998</v>
     <v>Beverages</v>
     <v>1 Monster Way, CORONA, CA, 92879-7101 US</v>
     <v>MNST</v>
     <v>Acciones</v>
     <v>MONSTER BEVERAGE CORPORATION (XNAS:MNST)</v>
-    <v>7726961</v>
+    <v>7727176</v>
     <v>9955571</v>
   </rv>
   <rv s="2">
@@ -10714,15 +10727,15 @@
     <v>164.13200000000001</v>
     <v>1.2746</v>
     <v>1.96</v>
-    <v>-1.7360000000000001E-3</v>
+    <v>3.509E-3</v>
     <v>1.2214000000000001E-2</v>
-    <v>-0.28199999999999997</v>
+    <v>0.56999999999999995</v>
     <v>95766405251</v>
     <v>160.47</v>
     <v>Airbnb, Inc. Opera una plataforma global para estancias y experiencias. El modelo de mercado de la Compañía conecta a anfitriones y huéspedes en línea o a través de dispositivos móviles para reservar espacios y experiencias en todo el mundo. La Compañía ha construido su plataforma para incorporar nuevos hosts, especialmente aquellos que anteriormente no habían considerado hosting. Se asocia con los anfitriones durante todo el proceso de configuración de su listado y les proporciona un conjunto de herramientas para administrar sus listados, incluyendo programación, merchandising, pagos integrados, soporte comunitario, etc. protección del anfitrión, orientación de precios y comentarios de las revisiones. Su sitio web y aplicaciones móviles ofrecen a sus huéspedes una manera de explorar una variedad de hogares y experiencias y una manera fácil de reservarlos. Su plataforma tecnológica impulsa su mercado de dos caras y permite su red global de anfitriones e invitados. Posee una cartera de marcas con protección en 220 países en los que opera para sus marcas principales, AIRBNB, y su logotipo de Belo.</v>
     <v>8200</v>
     <v>XNAS</v>
-    <v>46297.846665289064</v>
+    <v>46297.869787800781</v>
     <v>Nasdaq Stock Market</v>
     <v>58</v>
     <v>164.91</v>
@@ -10734,13 +10747,13 @@
     <v>AIRBNB, INC.</v>
     <v>36.933500000000002</v>
     <v>162.43</v>
-    <v>162.148</v>
+    <v>163</v>
     <v>Software &amp; IT Services</v>
     <v>888 Brannan St., SAN FRANCISCO, CA, 94103 US</v>
     <v>ABNB</v>
     <v>Acciones</v>
     <v>AIRBNB, INC. (XNAS:ABNB)</v>
-    <v>3362364</v>
+    <v>3362479</v>
     <v>5078272</v>
   </rv>
   <rv s="2">
@@ -10825,7 +10838,7 @@
     <v>Veralto Corporation proporciona soluciones tecnológicas esenciales que monitorean, mejoran y protegen los recursos clave en todo el mundo. Sus segmentos incluyen Calidad del Agua (WQ) y Calidad e Innovación del Producto (PQI). WQ Segment ofrece carteras de análisis de agua y soluciones de tratamiento de agua diferenciadas que permiten el suministro de agua potable segura por parte de empresas públicas y privadas. Bajo sus marcas Hach, Trojan Technologies, ChemTreat y otras marcas WQ reconocidas mundialmente, proporciona instrumentación de precisión y tecnologías avanzadas de tratamiento de agua en las que sus clientes confían para medir, analizar y tratar el agua en aplicaciones residenciales, comerciales, municipales, industriales, de investigación y de recursos naturales. El segmento PQI proporciona un conjunto de soluciones esenciales para los propietarios de marcas y las empresas de bienes de consumo envasados. Bajo sus marcas Videojet, Linx, Esko, X-Rite, Pantone y otras marcas PQI reconocidas a nivel mundial, proporciona marcado y codificación, así como embalaje e instrumentación de color y consumibles relacionados.</v>
     <v>17000</v>
     <v>XNYS</v>
-    <v>46297.847223298435</v>
+    <v>46297.872238414064</v>
     <v>New York Stock Exchange</v>
     <v>95.37</v>
     <v>107.9</v>
@@ -10834,7 +10847,7 @@
     <v>USD</v>
     <v>VERALTO CORPORATION</v>
     <v>VERALTO CORPORATION</v>
-    <v>23.869399999999999</v>
+    <v>23.846699999999998</v>
     <v>94.69</v>
     <v>94.68</v>
     <v>Professional &amp; Commercial Services</v>
@@ -10842,7 +10855,7 @@
     <v>VLTO</v>
     <v>Acciones</v>
     <v>VERALTO CORPORATION (XNYS:VLTO)</v>
-    <v>1536849</v>
+    <v>1620749</v>
     <v>1756177</v>
   </rv>
   <rv s="2">
@@ -10895,7 +10908,7 @@
     <v>Acciones</v>
     <v>Legrand SA (XPAR:LR)</v>
     <v>561126</v>
-    <v>599580</v>
+    <v>613070</v>
   </rv>
   <rv s="2">
     <v>67</v>
@@ -11041,7 +11054,7 @@
     <v>Meta Platforms, Inc. Está construyendo conexiones humanas, impulsadas por inteligencia artificial y tecnologías inmersivas. Los productos de la Compañía permiten a las personas conectarse y compartir con amigos y familiares a través de dispositivos móviles, computadoras personales, auriculares de realidad virtual (VR) y realidad mixta (MR), realidad aumentada (AR) y wearables. También ayuda a las personas a descubrir y aprender sobre lo que está sucediendo en el mundo que les rodea, permitiendo a las personas compartir sus experiencias, ideas, fotos, videos y otros contenidos con audiencias que van desde sus familiares y amigos más cercanos hasta el público en general. Los segmentos de la compañía incluyen Family of Apps (FOA) y Reality Labs (RL). El segmento FOA incluye Facebook, Instagram, Messenger, WhatsApp e hilos. El segmento de RL incluye su hardware, software y contenido de consumo relacionado con la realidad virtual, aumentada y mixta. Sus ofertas de productos en realidad virtual incluyen sus dispositivos Meta Quest, así como software y contenido disponible a través de la Tienda Meta Horizon.</v>
     <v>75472</v>
     <v>XNAS</v>
-    <v>46297.855588032035</v>
+    <v>46297.872355126565</v>
     <v>Nasdaq Stock Market</v>
     <v>75</v>
     <v>741.58</v>
@@ -11059,7 +11072,7 @@
     <v>META</v>
     <v>Acciones</v>
     <v>META PLATFORMS, INC. (XNAS:META)</v>
-    <v>12864675</v>
+    <v>12870985</v>
     <v>22283513</v>
   </rv>
   <rv s="2">
@@ -11081,17 +11094,17 @@
     <v>3</v>
     <v>4</v>
     <v>Finance</v>
-    <v>5</v>
+    <v>17</v>
     <v>XNYS</v>
     <v>897635600</v>
     <v>2021</v>
     <v>91.71</v>
     <v>1.7305999999999999</v>
-    <v>-0.98</v>
+    <v>-0.95</v>
     <v>4.2120000000000005E-3</v>
-    <v>-1.0741000000000001E-2</v>
+    <v>-1.0411999999999999E-2</v>
     <v>0.38030000000000003</v>
-    <v>81020589256</v>
+    <v>81047518324</v>
     <v>91.24</v>
     <v>KKR &amp; Co. Inc. Es una empresa de inversión global que ofrece gestión alternativa de activos, mercados de capital y soluciones de seguros. Los segmentos de la Compañía incluyen Gestión de Activos, Seguros y Holdings Estratégicos. El segmento de gestión de activos ofrece una gama de servicios de gestión de inversiones a fondos de inversión, vehículos y cuentas y proporciona servicios de mercados de capitales a empresas de cartera y terceros. El segmento de Gestión de Activos incluye cinco líneas de negocio: Capital Privado, Activos Inmobiliarios, Estrategias de Crédito y Líquido, Mercados de Capitales y Actividades Principales. El segmento de seguros es operado por Global Atlantic, que es una compañía de seguros de vida y jubilación de los Estados Unidos que ofrece un conjunto de productos de protección, herencia y ahorro y soluciones de reaseguro a clientes en los mercados individuales e institucionales. Global Atlantic ofrece anualidades de tasa fija a individuos y otras. El segmento Estratégico Holdings representa su participación en su estrategia básica de capital riesgo.</v>
     <v>5043</v>
@@ -11106,8 +11119,8 @@
     <v>USD</v>
     <v>KKR &amp; CO. INC.</v>
     <v>KKR &amp; CO. INC.</v>
-    <v>28.7745</v>
-    <v>90.26</v>
+    <v>28.784099999999999</v>
+    <v>90.29</v>
     <v>90.670299999999997</v>
     <v>Investment Banking &amp; Investment Services</v>
     <v>30 Hudson Yards, NEW YORK, NY, 10001 US</v>
@@ -11124,17 +11137,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=brh6oc&amp;q=XNYS%3aNET&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="8">
+  <rv s="1">
     <v>es-ES</v>
     <v>brh6oc</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>32</v>
-    <v>33</v>
+    <v>0</v>
+    <v>1</v>
     <v>CLOUDFLARE, INC. (XNYS:NET)</v>
     <v>3</v>
-    <v>34</v>
+    <v>4</v>
     <v>Finance</v>
     <v>5</v>
     <v>XNYS</v>
@@ -11143,15 +11156,15 @@
     <v>351.8</v>
     <v>1.3416999999999999</v>
     <v>-2.08</v>
-    <v>-2.0049999999999999E-4</v>
+    <v>-7.7349999999999999E-4</v>
     <v>-5.9259999999999998E-3</v>
-    <v>-7.0000000000000007E-2</v>
+    <v>-0.27</v>
     <v>124243328924</v>
     <v>351</v>
     <v>Cloudflare, Inc. Es una compañía de conectividad en la nube. Su conjunto completo de productos consiste en sus servicios de sitio web y aplicaciones para ofrecer seguridad, rendimiento y confiabilidad para los sitios web, aplicaciones e interfaces de programación de aplicaciones (API) de una organización; su plataforma Secure Access Service Edge (SASE), que contiene su conjunto de soluciones Zero Trust y servicios de red para ayudar a garantizar que el tráfico de entrada y salida de la red interna y los dispositivos de una organización se verifique y autorice, así como para conectar de forma segura centros de datos, servicios en la nube y sucursales a una organización con su Connectivity Cloud; sus soluciones basadas en desarrolladores para crear e implementar aplicaciones sin servidor con escala, rendimiento, seguridad y confiabilidad, y sus ofertas para consumidores. Sus ofertas de productos de seguridad de sitios web y aplicaciones incluyen firewall de aplicaciones web, gestión de bots, protección de denegación de servicio distribuida, seguridad de API, cifrado SSL/TLS, administración de scripts y centro de seguridad.</v>
     <v>5483</v>
     <v>XNYS</v>
-    <v>46297.854603344531</v>
+    <v>46297.870821515622</v>
     <v>New York Stock Exchange</v>
     <v>81</v>
     <v>354.58</v>
@@ -11161,14 +11174,15 @@
     <v>USD</v>
     <v>CLOUDFLARE, INC.</v>
     <v>CLOUDFLARE, INC.</v>
+    <v>0</v>
     <v>348.92</v>
-    <v>349</v>
+    <v>348.8</v>
     <v>Software &amp; IT Services</v>
     <v>101 Townsend St, SAN FRANCISCO, CA, 94107-1934 US</v>
     <v>NET</v>
     <v>Acciones</v>
     <v>CLOUDFLARE, INC. (XNYS:NET)</v>
-    <v>2832727</v>
+    <v>2833977</v>
     <v>3150420</v>
   </rv>
   <rv s="2">
@@ -11197,15 +11211,15 @@
     <v>269.5</v>
     <v>1.1780999999999999</v>
     <v>3.95</v>
-    <v>-7.2249999999999994E-4</v>
+    <v>1.4809999999999999E-4</v>
     <v>1.4844999999999999E-2</v>
-    <v>-0.1951</v>
+    <v>0.04</v>
     <v>276503407400</v>
     <v>266.08999999999997</v>
     <v>CrowdStrike Holdings, Inc. Es una compañía global de ciberseguridad que proporciona protección en la nube para endpoints, cargas de trabajo en la nube, identidad y datos. Su plataforma Falcon está diseñada para la consolidación de la ciberseguridad, diseñada específicamente para detener las brechas. Las plataformas recopilan e integran datos de toda la empresa, incluidos puntos finales, cargas de trabajo en la nube, identidades y fuentes de terceros. Ofrece 29 módulos en la nube en su plataforma Falcon a través de un modelo basado en suscripción de software como servicio (SaaS) que abarca múltiples mercados grandes, incluyendo seguridad de endpoints corporativos y cargas de trabajo en la nube, servicios de seguridad gestionada, gestión de operaciones de tecnología de la información (TI), protección de identidades, gestión de información de seguridad de próxima generación y gestión de eventos (SIEM) y gestión de registros, servicios de inteligencia contra amenazas, protección de datos, gestión de posturas de seguridad SaaS, automatización y respuesta (SOAR) y automatización de flujo de trabajo impulsada por inteligencia artificial, entre otros.</v>
     <v>11706</v>
     <v>XNAS</v>
-    <v>46297.854815392966</v>
+    <v>46297.87140755781</v>
     <v>Nasdaq Stock Market</v>
     <v>84</v>
     <v>273.5351</v>
@@ -11217,13 +11231,13 @@
     <v>CROWDSTRIKE HOLDINGS, INC.</v>
     <v>4737.5438999999997</v>
     <v>270.04000000000002</v>
-    <v>269.8449</v>
+    <v>270.08</v>
     <v>Software &amp; IT Services</v>
     <v>206 E. 9TH STREET, SUITE 1400, AUSTIN, TX, 78701 US</v>
     <v>CRWD</v>
     <v>Acciones</v>
     <v>CROWDSTRIKE HOLDINGS, INC. (XNAS:CRWD)</v>
-    <v>5824659</v>
+    <v>5828935</v>
     <v>12005594</v>
   </rv>
   <rv s="2">
@@ -11252,15 +11266,15 @@
     <v>338.1</v>
     <v>1.2044999999999999</v>
     <v>5.42</v>
-    <v>-7.3450000000000002E-4</v>
+    <v>-1.322E-3</v>
     <v>1.6182000000000002E-2</v>
-    <v>-0.25</v>
+    <v>-0.45</v>
     <v>4162480500000</v>
     <v>334.93</v>
     <v>Alphabet Inc. Es una compañía holding. Los segmentos de la Compañía incluyen Google Services, Google Cloud y otras apuestas. El segmento de Servicios de Google incluye productos y servicios como anuncios, Android, Chrome, dispositivos, Google Maps, Google Maps, etc. Google Play, Búsqueda y YouTube. El segmento de Google Cloud incluye servicios de infraestructura y plataforma, herramientas de colaboración y otros servicios para clientes empresariales. Su otro segmento de apuestas se dedica a la venta de servicios relacionados con la salud y servicios de Internet. Google Cloud ofrece servicios en la nube listos para la empresa, incluidos Google Cloud Platform y Google Workspace. Google Cloud Platform proporciona acceso a soluciones como las ofertas de inteligencia artificial (IA), incluida su infraestructura de IA, la plataforma Vertex AI y Gemini para Google Cloud; ciberseguridad y datos y análisis. Google Workspace incluye herramientas de comunicación y colaboración basadas en la nube para empresas, como Calendar, Gmail, Docs, Drive, y reunirse.</v>
     <v>198933</v>
     <v>XNAS</v>
-    <v>46297.855750786715</v>
+    <v>46297.872366875003</v>
     <v>Nasdaq Stock Market</v>
     <v>87</v>
     <v>342.78</v>
@@ -11272,29 +11286,29 @@
     <v>ALPHABET INC.</v>
     <v>17.1083</v>
     <v>340.35</v>
-    <v>340.1</v>
+    <v>339.9</v>
     <v>Software &amp; IT Services</v>
     <v>1600 Amphitheatre Parkway, MOUNTAIN VIEW, CA, 94043 US</v>
     <v>GOOG</v>
     <v>Acciones</v>
     <v>ALPHABET INC. (XNAS:GOOG)</v>
-    <v>17373579</v>
+    <v>17381365</v>
     <v>17655484</v>
   </rv>
   <rv s="2">
     <v>88</v>
   </rv>
-  <rv s="9">
+  <rv s="8">
     <v>es-ES</v>
     <v>cjjy9c</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>35</v>
-    <v>36</v>
+    <v>32</v>
+    <v>33</v>
     <v>Abb Ltd (XSWX:ABBNE)</v>
     <v>27</v>
-    <v>37</v>
+    <v>34</v>
     <v>Finance</v>
     <v>15</v>
     <v>XSWX</v>
@@ -11344,17 +11358,17 @@
     <v>3</v>
     <v>4</v>
     <v>Finance</v>
-    <v>5</v>
+    <v>17</v>
     <v>XNYS</v>
     <v>192852500</v>
     <v>2010</v>
     <v>284.01</v>
     <v>0.9022</v>
-    <v>-1.43</v>
+    <v>-1.3</v>
     <v>0</v>
-    <v>-5.0629999999999998E-3</v>
+    <v>-4.6020000000000002E-3</v>
     <v>0</v>
-    <v>54197338074</v>
+    <v>54222408900</v>
     <v>282.45999999999998</v>
     <v>Garmin Ltd. (Garmin) es una entidad con sede en Suiza. La Compañía y sus filiales ofrecen sistemas de posicionamiento global (GPS) y dispositivos y aplicaciones inalámbricas. La Compañía opera a través de cinco segmentos: Fitness, outdoor, aviación, marina y auto. Ofrece una gama de productos de navegación automática, así como una gama de productos y aplicaciones diseñados para el mercado de GPS móvil. Ofrece Handhelds al aire libre, dispositivos portables, dispositivos de golf y dispositivos de seguimiento de perros y entrenamiento / obediencia de mascotas. Garmin ofrece varios productos diseñados para su uso en el seguimiento de fitness y actividad. El segmento de negocios de aviación de la compañía es un proveedor de soluciones para fabricantes de aeronaves, propietarios y operadores de aeronaves existentes, así como clientes militares y gubernamentales, y sirve a una gama de aeronaves, incluyendo aviones de transporte, aviación de negocios, aviación general, deportes experimentales / ligeros, etc. helicópteros, vehículos pilotados opcionalmente y vehículos aéreos no tripulados. La compañía opera en todo el mundo.</v>
     <v>23000</v>
@@ -11369,8 +11383,8 @@
     <v>USD</v>
     <v>Garmin Ltd.</v>
     <v>Garmin Ltd.</v>
-    <v>28.9817</v>
-    <v>281.02999999999997</v>
+    <v>28.995100000000001</v>
+    <v>281.16000000000003</v>
     <v>281.16000000000003</v>
     <v>Communications &amp; Networking</v>
     <v>Muehlentalstrasse 2, SCHAFFHAUSEN, SCHAFFHAUSEN, 8200 CH</v>
@@ -11494,17 +11508,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=amft3m&amp;q=BMEX%3aCBAV&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="10">
+  <rv s="9">
     <v>es-ES</v>
     <v>amft3m</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>38</v>
-    <v>39</v>
+    <v>35</v>
+    <v>36</v>
     <v>CLINICA BAVIERA S.A (BMEX:CBAV)</v>
     <v>3</v>
-    <v>40</v>
+    <v>37</v>
     <v>Finance</v>
     <v>15</v>
     <v>BMEX</v>
@@ -11564,15 +11578,15 @@
     <v>236.05500000000001</v>
     <v>2.1901000000000002</v>
     <v>3.09</v>
-    <v>3.8470000000000003E-5</v>
+    <v>-3.4200000000000002E-4</v>
     <v>1.3385000000000001E-2</v>
-    <v>8.9999999999999993E-3</v>
+    <v>-0.08</v>
     <v>5638195000000</v>
     <v>230.86</v>
     <v>NVIDIA Corporation es una empresa de infraestructura de computación completa. La Compañía se dedica a la computación acelerada para ayudar a resolver los problemas computacionales desafiantes. Los segmentos de la Compañía incluyen Compute &amp; Networking y Gráficos. El segmento Compute &amp; Networking incluye sus plataformas de computación acelerada de centros de datos y soluciones y software de inteligencia artificial (IA); redes; plataformas automotrices y soluciones de vehículos autónomos y eléctricos; Jetson para robótica y otras plataformas integradas, y servicios de computación en la nube DGX. El segmento de gráficos incluye GPU GeForce para juegos y PC, el servicio de streaming de juegos GeForce NOW e infraestructura relacionada, y soluciones para plataformas de juegos; GPU Quadro/NVIDIA RTX para gráficos de estaciones de trabajo empresariales; software de GPU virtual para computación visual y virtual basada en la nube; plataformas automotrices para sistemas de infoentretenimiento y software Omniverse Enterprise para construir y operar aplicaciones industriales de IA y gemelas digitales.</v>
     <v>42000</v>
     <v>XNAS</v>
-    <v>46297.855726365626</v>
+    <v>46297.872427777344</v>
     <v>Nasdaq Stock Market</v>
     <v>104</v>
     <v>237.88</v>
@@ -11584,13 +11598,13 @@
     <v>NVIDIA CORPORATION</v>
     <v>29.573899999999998</v>
     <v>233.95</v>
-    <v>233.959</v>
+    <v>233.87</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>2788 San Tomas Expressway, SANTA CLARA, CA, 95051 US</v>
     <v>NVDA</v>
     <v>Acciones</v>
     <v>NVIDIA CORPORATION (XNAS:NVDA)</v>
-    <v>134361543</v>
+    <v>134462193</v>
     <v>123376907</v>
   </rv>
   <rv s="2">
@@ -11671,15 +11685,15 @@
     <v>465.64</v>
     <v>1.4258999999999999</v>
     <v>13.67</v>
-    <v>-5.4870000000000006E-4</v>
+    <v>-8.4610000000000002E-4</v>
     <v>2.9769E-2</v>
-    <v>-0.25940000000000002</v>
+    <v>-0.4</v>
     <v>2452527960380</v>
     <v>459.2</v>
     <v>Taiwan Semiconductor Manufacturing Co Ltd es una empresa con sede en Taiwán dedicada principalmente a la prestación de servicios de fabricación de circuitos integrados. Los servicios integrados de fabricación de circuitos incluyen tecnología de proceso, tecnología de proceso especial, soporte del ecosistema de diseño, tecnología de máscara, embalaje avanzado 3DFabricTM y servicios de tecnología de apilamiento de silicio. La compañía ha completado la transferencia y la producción en masa de la tecnología 5nm, y se dedica a la investigación y desarrollo de la tecnología de proceso 3nm y la tecnología de proceso 2nm. La gama de aplicaciones de productos cubre toda la industria de aplicaciones electrónicas, incluyendo computadoras personales y productos periféricos, productos de aplicaciones de información, productos de sistemas de comunicación cableados e inalámbricos, servidores y centros de datos.</v>
     <v>52045</v>
     <v>XNYS</v>
-    <v>46297.855446399997</v>
+    <v>46297.87221554375</v>
     <v>New York Stock Exchange</v>
     <v>110</v>
     <v>474.79</v>
@@ -11691,13 +11705,13 @@
     <v>Taiwan Semiconductor Manufacturing Company Limited</v>
     <v>34.393500000000003</v>
     <v>472.87</v>
-    <v>472.5206</v>
+    <v>472.38</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>No.8, Li-Hsin 6th Road, Hsinchu Science Park, HSINCHU, HSINCHU, 300 TW</v>
     <v>TSM</v>
     <v>Acciones</v>
     <v>Taiwan Semiconductor Manufacturing Company Limited (XNYS:TSM)</v>
-    <v>9720360</v>
+    <v>9722368</v>
     <v>9752833</v>
   </rv>
   <rv s="2">
@@ -11726,15 +11740,15 @@
     <v>491.2</v>
     <v>1.5275000000000001</v>
     <v>-18.545000000000002</v>
-    <v>1.227E-3</v>
+    <v>3.2600000000000003E-3</v>
     <v>-3.7738999999999995E-2</v>
-    <v>0.57999999999999996</v>
+    <v>1.5417000000000001</v>
     <v>97187874141</v>
     <v>491.4</v>
     <v>Spotify Technology SA es una empresa con sede en Luxemburgo que ofrece servicios de música digital en streaming. La Compañía permite a los usuarios descubrir nuevos lanzamientos, que incluyen los últimos singles y álbumes; listas de reproducción, que incluye listas de reproducción preparadas por fanáticos de la música y expertos, y más de millones de canciones para que los usuarios puedan reproducir sus favoritos, descubrir nuevas pistas y construir una colección personalizada. Sus usuarios pueden seleccionar Spotify Free, que incluye solo reproducción aleatoria o Spotify Premium, que abarca una gama de características, como reproducción aleatoria, publicidad gratuita, saltos ilimitados, escuchar sin conexión, reproducir cualquier pista y audio. La Compañía opera a través de una serie de subsidiarias, incluyendo Spotify LTD y está presente en más de 20 países. Su servicio ofrece una experiencia de escucha de música sin pausas comerciales.</v>
     <v>7287</v>
     <v>XNYS</v>
-    <v>46297.855739814062</v>
+    <v>46297.867253471872</v>
     <v>New York Stock Exchange</v>
     <v>113</v>
     <v>492.505</v>
@@ -11746,13 +11760,13 @@
     <v>Spotify Technology S.A.</v>
     <v>26.126799999999999</v>
     <v>472.85500000000002</v>
-    <v>473.47</v>
+    <v>474.43169999999998</v>
     <v>Software &amp; IT Services</v>
     <v>33, Boulevard Prince Henri, LUXEMBOURG, 1724 LU</v>
     <v>SPOT</v>
     <v>Acciones</v>
     <v>Spotify Technology S.A. (XNYS:SPOT)</v>
-    <v>1890869</v>
+    <v>1891343</v>
     <v>1450469</v>
   </rv>
   <rv s="2">
@@ -11762,19 +11776,19 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=ajg6ec&amp;q=XMIL%3aPRY&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="10">
+  <rv s="9">
     <v>es-ES</v>
     <v>ajg6ec</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>38</v>
-    <v>39</v>
+    <v>35</v>
+    <v>36</v>
     <v>Prysmian S.p.A. (XMIL:PRY)</v>
     <v>3</v>
-    <v>40</v>
+    <v>37</v>
     <v>Finance</v>
-    <v>41</v>
+    <v>38</v>
     <v>XMIL</v>
     <v>308861600</v>
     <v>126.75</v>
@@ -11880,7 +11894,7 @@
     <v>3</v>
     <v>14</v>
     <v>Finance</v>
-    <v>41</v>
+    <v>38</v>
     <v>XMIL</v>
     <v>1231268000</v>
     <v>2020</v>
@@ -12030,19 +12044,19 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=ajgoa2&amp;q=XMIL%3aTGYM&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="10">
+  <rv s="9">
     <v>es-ES</v>
     <v>ajgoa2</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>38</v>
-    <v>39</v>
+    <v>35</v>
+    <v>36</v>
     <v>Technogym S.p.A. (XMIL:TGYM)</v>
     <v>3</v>
-    <v>40</v>
+    <v>37</v>
     <v>Finance</v>
-    <v>41</v>
+    <v>38</v>
     <v>XMIL</v>
     <v>201327500</v>
     <v>13.28</v>
@@ -12081,17 +12095,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=amg4gh&amp;q=BMEX%3aVID&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="10">
+  <rv s="9">
     <v>es-ES</v>
     <v>amg4gh</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>38</v>
-    <v>39</v>
+    <v>35</v>
+    <v>36</v>
     <v>VIDRALA, S.A. (BMEX:VID)</v>
     <v>3</v>
-    <v>40</v>
+    <v>37</v>
     <v>Finance</v>
     <v>15</v>
     <v>BMEX</v>
@@ -12142,9 +12156,9 @@
     <v>1</v>
     <v>Triple Flag Prec (XTSE:TFPM)</v>
     <v>3</v>
-    <v>42</v>
+    <v>39</v>
     <v>Finance</v>
-    <v>43</v>
+    <v>40</v>
     <v>XTSE</v>
     <v>206003000</v>
     <v>2019</v>
@@ -12177,7 +12191,7 @@
     <v>TFPM</v>
     <v>Acciones</v>
     <v>Triple Flag Prec (XTSE:TFPM)</v>
-    <v>103900</v>
+    <v>103856</v>
     <v>166370</v>
   </rv>
   <rv s="2">
@@ -12206,15 +12220,15 @@
     <v>67.599999999999994</v>
     <v>1.6013999999999999</v>
     <v>-0.79</v>
-    <v>5.5620000000000008E-4</v>
+    <v>8.7529999999999997E-4</v>
     <v>-1.1642999999999999E-2</v>
-    <v>3.73E-2</v>
+    <v>5.8700000000000002E-2</v>
     <v>279233749340</v>
     <v>67.849999999999994</v>
     <v>Netflix, Inc. Es un proveedor de servicios de entretenimiento. La Compañía adquiere, concede licencias y produce contenido, incluida la programación original. Ofrece membresías pagadas en más de 190 países que ofrecen series de televisión (TV), películas y juegos en una variedad de géneros e idiomas. Permite a los miembros jugar, pausar y reanudar la mirada tanto como quieran, en cualquier momento y en cualquier lugar, y puede cambiar sus planes en cualquier momento. La Compañía ofrece a los miembros la posibilidad de recibir contenido en streaming a través de una serie de dispositivos conectados a Internet, incluidos televisores, reproductores de video digital, decodificadores de TV y dispositivos móviles. Se dedica a escalar su servicio de streaming, como la introducción de juegos y publicidad en su servicio, así como ofrecer programación en vivo. Está desarrollando tecnología y utilizando computación en la nube de terceros, tecnología y otros servicios. La Compañía también se dedica a escalar sus propias operaciones de estudio para producir contenido original.</v>
     <v>16000</v>
     <v>XNAS</v>
-    <v>46297.855677649997</v>
+    <v>46297.872411388278</v>
     <v>Nasdaq Stock Market</v>
     <v>140</v>
     <v>67.87</v>
@@ -12226,13 +12240,13 @@
     <v>NETFLIX, INC.</v>
     <v>21.1266</v>
     <v>67.06</v>
-    <v>67.097300000000004</v>
+    <v>67.118700000000004</v>
     <v>Software &amp; IT Services</v>
     <v>121 Albright Way, LOS GATOS, CA, 95032 US</v>
     <v>NFLX</v>
     <v>Acciones</v>
     <v>NETFLIX, INC. (XNAS:NFLX)</v>
-    <v>38274522</v>
+    <v>38310797</v>
     <v>33271285</v>
   </rv>
   <rv s="2">
@@ -12261,15 +12275,15 @@
     <v>32.552999999999997</v>
     <v>1.0439000000000001</v>
     <v>-1.2549999999999999</v>
-    <v>-1.178E-3</v>
+    <v>-8.8279999999999999E-4</v>
     <v>-3.5704E-2</v>
-    <v>-3.9899999999999998E-2</v>
+    <v>-2.9899999999999999E-2</v>
     <v>50283198605</v>
     <v>35.15</v>
     <v>NIKE, Inc. Se dedica al diseño, comercialización y distribución de calzado deportivo, ropa, equipos y accesorios y servicios para actividades deportivas y de fitness. Los segmentos operativos de la compañía incluyen América del Norte, Europa, Oriente Medio y África (EMEA), Gran China y Asia Pacífico y América Latina (APLA). Vende una línea de equipos y accesorios bajo la marca NIKE, incluyendo bolsos, calcetines, bolas deportivas, gafas, relojes, dispositivos digitales, murciélagos, guantes, equipos de protección y otros equipos diseñados para actividades deportivas. También diseña productos específicamente para la marca Jordan y Converse. La marca Jordan diseña, distribuye y otorga licencias de calzado deportivo y casual, ropa y accesorios principalmente centrados en el rendimiento y la cultura del baloncesto utilizando la marca Jumpman. La Compañía también diseña, distribuye y otorga licencias de zapatillas de deporte casuales, ropa y accesorios bajo las marcas registradas Chuck Taylor, All Star, One Star, Star Chevron y Jack Purcell.</v>
     <v>73000</v>
     <v>XNYS</v>
-    <v>46297.855665578129</v>
+    <v>46297.872373911719</v>
     <v>New York Stock Exchange</v>
     <v>143</v>
     <v>33.97</v>
@@ -12281,13 +12295,13 @@
     <v>NIKE, INC.</v>
     <v>16.245699999999999</v>
     <v>33.895000000000003</v>
-    <v>33.830100000000002</v>
+    <v>33.8401</v>
     <v>Textiles &amp; Apparel</v>
     <v>One Bowerman Dr, BEAVERTON, OR, 97005-6453 US</v>
     <v>NKE</v>
     <v>Acciones</v>
     <v>NIKE, INC. (XNYS:NKE)</v>
-    <v>141755766</v>
+    <v>141936094</v>
     <v>35960177</v>
   </rv>
   <rv s="2">
@@ -12297,17 +12311,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=amwwgh&amp;q=XSTO%3aMIPS&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="11">
+  <rv s="10">
     <v>es-ES</v>
     <v>amwwgh</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>44</v>
-    <v>45</v>
+    <v>41</v>
+    <v>42</v>
     <v>MIPS (XSTO:MIPS)</v>
     <v>3</v>
-    <v>46</v>
+    <v>43</v>
     <v>Finance</v>
     <v>22</v>
     <v>XSTO</v>
@@ -12362,17 +12376,17 @@
     <v>3</v>
     <v>4</v>
     <v>Finance</v>
-    <v>5</v>
+    <v>17</v>
     <v>XNYS</v>
     <v>193452700</v>
     <v>2024</v>
     <v>224.18</v>
     <v>1.1184000000000001</v>
-    <v>1.88</v>
+    <v>1.84</v>
     <v>0</v>
-    <v>8.4880000000000008E-3</v>
+    <v>8.3070000000000001E-3</v>
     <v>0</v>
-    <v>43211529599</v>
+    <v>43203791491</v>
     <v>221.49</v>
     <v>Ferguson Enterprises Inc. Es un distribuidor de valor agregado que sirve a profesionales especializados en el mercado de la construcción residencial y no residencial de América del Norte. Los segmentos geográficos de la Compañía incluyen Estados Unidos y Canadá. La Compañía ofrece una amplia gama de productos y servicios, tales como plomería, calefacción, ventilación y aire acondicionado (HVAC), electrodomésticos e iluminación para tuberías, válvulas y accesorios (PVF), soluciones de agua y aguas residuales, y más. Se vende a través de una red común de centros de distribución, sucursales, servicio de mostrador y asociados de ventas especializados, consultores de showroom y canales de comercio electrónico. La compañía sirve a diversas industrias, tales como plomería, HVAC, comercial / mecánica, suministro de instalaciones, fuego y fabricación, industrial, constructor, obras de agua. Las marcas de la compañía incluyen Armateck, Durastar, FNW, National Fire Products, Pollardwater, PROFLO, PROSELECT, Raptor, Hardware de firma y Westcraft.</v>
     <v>35000</v>
@@ -12387,8 +12401,8 @@
     <v>USD</v>
     <v>FERGUSON ENTERPRISES INC.</v>
     <v>FERGUSON ENTERPRISES INC.</v>
-    <v>21.980699999999999</v>
-    <v>223.37</v>
+    <v>21.976800000000001</v>
+    <v>223.33</v>
     <v>223.33</v>
     <v>Homebuilding &amp; Construction Supplies</v>
     <v>751 Lakefront Commons, NEWPORT NEWS, VA, 23606 US</v>
@@ -12424,15 +12438,15 @@
     <v>24.92</v>
     <v>0.60040000000000004</v>
     <v>0.38</v>
-    <v>-3.9899999999999999E-4</v>
+    <v>-7.9810000000000005E-4</v>
     <v>1.5403E-2</v>
-    <v>-0.01</v>
+    <v>-0.02</v>
     <v>8718629955</v>
     <v>24.67</v>
     <v>SentinelOne, Inc. Es un proveedor de ciberseguridad impulsado por inteligencia artificial (IA). La Plataforma Singularity de la compañía ofrece capacidades autónomas de prevención, detección, respuesta y administración de exposición de amenazas impulsadas por IA en los endpoints, cargas de trabajo en la nube y credenciales de identidad de una organización. La plataforma Singularity de la compañía ingiere, correlaciona y consulta petabytes de datos estructurados y no estructurados de una miríada de fuentes externas e internas dispares en constante expansión en tiempo real. Sus modelos de IA distribuida se ejecutan tanto localmente en cada endpoint y cada carga de trabajo en la nube, así como en su plataforma en la nube. La compañía a través de PingSafe Pte. Ltd. (PingSafe), que es una plataforma de protección de aplicaciones nativa en la nube (CNAPP) para reforzar su paquete de productos de seguridad en la nube. Al agregar CNAPP de PingSafe a su Cloud Workload Security (CWS), proporciona a las empresas una cobertura de seguridad en la nube integral que impulsa la seguridad, la postura mejorada y la protección autónoma.</v>
     <v>2800</v>
     <v>XNYS</v>
-    <v>46297.85520537031</v>
+    <v>46297.867636875002</v>
     <v>New York Stock Exchange</v>
     <v>152</v>
     <v>25.75</v>
@@ -12444,13 +12458,13 @@
     <v>SENTINELONE, INC.</v>
     <v>0</v>
     <v>25.05</v>
-    <v>25.05</v>
+    <v>25.04</v>
     <v>Software &amp; IT Services</v>
     <v>444 Castro Street, Suite 400, MOUNTAIN VIEW, CA, 94041 US</v>
     <v>S</v>
     <v>Acciones</v>
     <v>SENTINELONE, INC. (XNYS:S)</v>
-    <v>11314587</v>
+    <v>11315947</v>
     <v>9622873</v>
   </rv>
   <rv s="2">
@@ -12479,15 +12493,15 @@
     <v>44.5</v>
     <v>1.4997</v>
     <v>0.06</v>
-    <v>-2.525E-5</v>
+    <v>-2.1551999999999998E-2</v>
     <v>1.379E-3</v>
-    <v>-1.1000000000000001E-3</v>
+    <v>-0.93879999999999997</v>
     <v>4437248112</v>
     <v>43.5</v>
     <v>Trex Company, Inc. Es un fabricante de terrazas alternativas de madera y barandillas residenciales y productos y accesorios para vivir al aire libre, comercializados bajo la marca Trex. El segmento de la compañía es Trex Residential. Sus categorías de productos incluyen cubiertas y accesorios, barandillas y cercas. Sus productos de terrazas están hechos en un proceso patentado que combina fibras de madera recuperadas y película de polietileno reciclado. Sus cubiertas y accesorios incluyen cubiertas Trex Signature, cubiertas Trex Transcend Lineage, cubiertas Trex Transcend, cubiertas Trex Select, cubiertas Trex Enhance, colección de sujetadores Trex Hideaway y sistema de iluminación exterior Trex DeckLighting. Su producto de decking Trex Transcend también se puede utilizar como revestimiento. Sus productos de barandilla incluyen barandilla Trex Signature X-Series, barandilla de aluminio Trex Signature, barandilla Trex Transcend, barandilla Trex Select, carril T Trex Select y barandilla Trex Enhance. Su producto compuesto de esgrima Trex Seclusions se ofrece a través de dos distribuidores especializados.</v>
     <v>1839</v>
     <v>XNYS</v>
-    <v>46297.846442823437</v>
+    <v>46297.866652603909</v>
     <v>New York Stock Exchange</v>
     <v>155</v>
     <v>44.96</v>
@@ -12497,15 +12511,15 @@
     <v>USD</v>
     <v>TREX COMPANY, INC.</v>
     <v>TREX COMPANY, INC.</v>
-    <v>25.708200000000001</v>
+    <v>25.673100000000002</v>
     <v>43.56</v>
-    <v>43.558900000000001</v>
+    <v>42.621200000000002</v>
     <v>Homebuilding &amp; Construction Supplies</v>
     <v>2500 TREX WAY, WINCHESTER, VA, 22601 US</v>
     <v>TREX</v>
     <v>Acciones</v>
     <v>TREX COMPANY, INC. (XNYS:TREX)</v>
-    <v>1563084</v>
+    <v>1563086</v>
     <v>1569141</v>
   </rv>
   <rv s="2">
@@ -12638,15 +12652,15 @@
     <v>27.75</v>
     <v>1.0061</v>
     <v>-0.66</v>
-    <v>1.5809999999999999E-3</v>
+    <v>2.9909999999999997E-3</v>
     <v>-2.4079000000000003E-2</v>
-    <v>4.2299999999999997E-2</v>
+    <v>0.08</v>
     <v>6768686250</v>
     <v>27.41</v>
     <v>Celsius Holdings, Inc. Se dedica al desarrollo, procesamiento, comercialización, venta y distribución de bebidas energéticas funcionales a una amplia gama de consumidores. El activo insignia de la Compañía, CELSIUS, se comercializa como un estilo de vida y bebida energética. Esta línea de productos viene en dos versiones: Una forma lista para beber y una forma de polvo en movimiento. También ofrece una nueva línea CELSIUS Essentials, disponible en latas de 16 onzas y una línea de hidratación de polvos con cero azúcar que se infunden con electrolitos y están disponibles en una variedad de sabores frutales. Los productos Celsius se ofrecen en canales minoristas a través de los Estados Unidos, incluyendo comestibles convencionales, naturales, conveniencia, fitness, etc. mercado masivo, especialidad de vitaminas y plataformas de comercio electrónico. Sus productos también se ofrecen en mercados seleccionados de Europa, Oriente Medio y la región de Asia-Pacífico. La formulación de su producto incluye ingredientes y suplementos como el té verde (EGCG), jengibre (de la raíz), calcio, cromo, vitaminas B y vitamina C.</v>
     <v>1497</v>
     <v>XNAS</v>
-    <v>46297.855420138279</v>
+    <v>46297.872410428128</v>
     <v>Nasdaq Stock Market</v>
     <v>164</v>
     <v>27.9</v>
@@ -12658,13 +12672,13 @@
     <v>CELSIUS HOLDINGS, INC.</v>
     <v>115.0043</v>
     <v>26.75</v>
-    <v>26.792300000000001</v>
+    <v>26.83</v>
     <v>Beverages</v>
     <v>2424 N. Federal Hwy, Suite 208, BOCA RATON, FL, 33431 US</v>
     <v>CELH</v>
     <v>Acciones</v>
     <v>CELSIUS HOLDINGS, INC. (XNAS:CELH)</v>
-    <v>8930419</v>
+    <v>8935162</v>
     <v>7099111</v>
   </rv>
   <rv s="2">
@@ -12726,17 +12740,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=bscvur&amp;q=XWBO%3aVRLA&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="12">
+  <rv s="11">
     <v>es-ES</v>
     <v>bscvur</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>47</v>
-    <v>48</v>
+    <v>44</v>
+    <v>45</v>
     <v>Verallia SA (XWBO:VRLA)</v>
     <v>3</v>
-    <v>49</v>
+    <v>46</v>
     <v>Finance</v>
     <v>15</v>
     <v>XWBO</v>
@@ -12772,14 +12786,14 @@
   <rv s="2">
     <v>171</v>
   </rv>
-  <rv s="13">
+  <rv s="12">
     <v>es-ES</v>
     <v>c8f4a2</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>50</v>
-    <v>51</v>
+    <v>47</v>
+    <v>48</v>
     <v>Kistos Holdings (XLON:KIST)</v>
     <v>27</v>
     <v>19</v>
@@ -12885,9 +12899,9 @@
     <v>1</v>
     <v>INTERNATIONAL PETROLEUM CORPORATION (XTSE:IPCO)</v>
     <v>3</v>
-    <v>52</v>
+    <v>49</v>
     <v>Finance</v>
-    <v>43</v>
+    <v>40</v>
     <v>XTSE</v>
     <v>112159300</v>
     <v>2017</v>
@@ -12995,9 +13009,9 @@
     <v>1</v>
     <v>Constellation Software Inc. (XTSE:CSU)</v>
     <v>3</v>
-    <v>42</v>
+    <v>39</v>
     <v>Finance</v>
-    <v>43</v>
+    <v>40</v>
     <v>XTSE</v>
     <v>21191530</v>
     <v>2002</v>
@@ -13012,7 +13026,7 @@
     <v>Constellation Software Inc. Es un proveedor de software y servicios con sede en Canadá para varias industrias. La Compañía adquiere, administra y construye negocios de software de mercado vertical (VMS) que proporcionan soluciones de software de misión crítica. Se dedica principalmente al desarrollo, instalación y personalización de software, así como en el suministro de servicios profesionales relacionados y soporte para clientes de todo el mundo. Sus servicios profesionales incluyen la instalación, implementación, capacitación y personalización de software y otros servicios. La Compañía vende licencias de software en las instalaciones tanto a perpetuo como a plazo especificado. Cuenta con seis grupos operativos, que dan servicio a clientes en más de 100 mercados diferentes en todo el mundo. Los seis grupos operativos incluyen Volaris, Harris, Topicus.com, Vela, Jonas, y Grupo Perseus. Opera oficinas en América del Norte, Europa Continental, Reino Unido, América del Sur, África, y Australia.</v>
     <v>64000</v>
     <v>XTSE</v>
-    <v>46297.833333333336</v>
+    <v>46297.84915509259</v>
     <v>Toronto Stock Exchange</v>
     <v>184</v>
     <v>3042.9749999999999</v>
@@ -13030,7 +13044,7 @@
     <v>CSU</v>
     <v>Acciones</v>
     <v>Constellation Software Inc. (XTSE:CSU)</v>
-    <v>51191</v>
+    <v>51123</v>
     <v>72480</v>
   </rv>
   <rv s="2">
@@ -13059,15 +13073,15 @@
     <v>68.239999999999995</v>
     <v>1.3212999999999999</v>
     <v>0.23</v>
-    <v>5.8730000000000002E-4</v>
+    <v>-1.6439999999999998E-4</v>
     <v>3.388E-3</v>
-    <v>0.04</v>
+    <v>-1.12E-2</v>
     <v>139118761600</v>
     <v>67.88</v>
     <v>Uber Technologies, Inc. Opera una plataforma tecnológica que utiliza redes y tecnología para impulsar el movimiento desde el punto A al punto B. Desarrolla y opera aplicaciones tecnológicas que soportan una variedad de ofertas en su plataforma (plataforma(s)). Sus segmentos incluyen Movilidad, Entrega y Carga. Los productos de movilidad conectan a los consumidores con conductores que ofrecen viajes en una variedad de vehículos, como automóviles, rickshaws de automóviles, motos, minibuses, etc. o taxis. Las ofertas de entrega permiten a los consumidores buscar y descubrir restaurantes locales, pedir una comida y recoger en el restaurante o hacer que se les entregue la comida. En ciertos mercados, el segmento de Entrega ofrece ofertas para la entrega de comestibles, alcohol y tiendas de conveniencia, así como otros productos seleccionados. El segmento de carga conecta a los transportistas con los transportistas en su plataforma, y ofrece a los transportistas por adelantado, precios y la capacidad de reservar un envío. El segmento de carga también incluye la gestión del transporte y otras ofertas de servicios logísticos.</v>
     <v>34000</v>
     <v>XNYS</v>
-    <v>46297.8552939</v>
+    <v>46297.872119930471</v>
     <v>New York Stock Exchange</v>
     <v>187</v>
     <v>68.47</v>
@@ -13077,15 +13091,15 @@
     <v>USD</v>
     <v>UBER TECHNOLOGIES, INC.</v>
     <v>UBER TECHNOLOGIES, INC.</v>
-    <v>14.950799999999999</v>
+    <v>14.9002</v>
     <v>68.11</v>
-    <v>68.150000000000006</v>
+    <v>68.098799999999997</v>
     <v>Software &amp; IT Services</v>
     <v>1725 3Rd Street, SAN FRANCISCO, CA, 94158 US</v>
     <v>UBER</v>
     <v>Acciones</v>
     <v>UBER TECHNOLOGIES, INC. (XNYS:UBER)</v>
-    <v>15476191</v>
+    <v>15498176</v>
     <v>17992531</v>
   </rv>
   <rv s="2">
@@ -13095,17 +13109,17 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=aodtkr&amp;q=XLON%3aSOM&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="14">
+  <rv s="13">
     <v>es-ES</v>
     <v>aodtkr</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>53</v>
-    <v>54</v>
+    <v>50</v>
+    <v>51</v>
     <v>Somero (XLON:SOM)</v>
     <v>3</v>
-    <v>55</v>
+    <v>52</v>
     <v>Finance</v>
     <v>29</v>
     <v>XLON</v>
@@ -13148,19 +13162,19 @@
     <v>https://www.bing.com/financeapi/forcetrigger?t=ajflbh&amp;q=XMIL%3aIP&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="10">
+  <rv s="9">
     <v>es-ES</v>
     <v>ajflbh</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>38</v>
-    <v>39</v>
+    <v>35</v>
+    <v>36</v>
     <v>Interpump Group S.p.A. (XMIL:IP)</v>
     <v>3</v>
-    <v>40</v>
+    <v>37</v>
     <v>Finance</v>
-    <v>41</v>
+    <v>38</v>
     <v>XMIL</v>
     <v>108879300</v>
     <v>35.82</v>
@@ -13247,17 +13261,17 @@
   <rv s="2">
     <v>197</v>
   </rv>
-  <rv s="15">
+  <rv s="14">
     <v>es-ES</v>
     <v>cg32pr</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>56</v>
-    <v>57</v>
+    <v>53</v>
+    <v>54</v>
     <v>Roko (XSTO:ROKO B)</v>
     <v>27</v>
-    <v>46</v>
+    <v>43</v>
     <v>Finance</v>
     <v>22</v>
     <v>XSTO</v>
@@ -13311,17 +13325,17 @@
     <v>3</v>
     <v>4</v>
     <v>Finance</v>
-    <v>5</v>
+    <v>17</v>
     <v>XNYS</v>
     <v>14922700</v>
     <v>1992</v>
     <v>83.21</v>
     <v>1.1626000000000001</v>
-    <v>1.24</v>
+    <v>1.1200000000000001</v>
     <v>0</v>
-    <v>1.5012000000000001E-2</v>
+    <v>1.3559000000000002E-2</v>
     <v>0</v>
-    <v>1251119168</v>
+    <v>1249328444</v>
     <v>82.6</v>
     <v>U.S. Physical Therapy, Inc. is an operator of outpatient physical therapy clinics and provider of industrial injury prevention services. It owns and/or manages 795 outpatient physical therapy clinics in 45 states. Its reportable segments include the Physical Therapy Operations segment and the Industrial Injury Prevention Services (IIP) segment. The Physical Therapy Operations segment consists of physical therapy, speech therapy and occupational therapy clinics and home-care physical and speech therapy practices that provide pre- and post-operative care and treatment for a variety of orthopedic-related disorders, sports-related injuries, and rehabilitation of injured workers. The IIP segment includes onsite services for clients’ employees, including injury prevention and rehabilitation, performance optimization, post-offer employment testing, functional capacity evaluations and ergonomic assessments. The majority of these services are contracted with and paid for directly by employers.</v>
     <v>4200</v>
@@ -13336,8 +13350,8 @@
     <v>USD</v>
     <v>US Physical</v>
     <v>US Physical</v>
-    <v>477.17700000000002</v>
-    <v>83.84</v>
+    <v>476.49400000000003</v>
+    <v>83.72</v>
     <v>83.72</v>
     <v>Healthcare Providers &amp; Services</v>
     <v>1300 West Sam Houston Parkway South, Suite 300, HOUSTON, TX, 77043 US</v>
@@ -13402,17 +13416,17 @@
   <rv s="2">
     <v>205</v>
   </rv>
-  <rv s="16">
+  <rv s="15">
     <v>es-ES</v>
     <v>dacqpr</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>58</v>
-    <v>59</v>
+    <v>55</v>
+    <v>56</v>
     <v>Vylor (XNYS:VYLR)</v>
     <v>27</v>
-    <v>60</v>
+    <v>57</v>
     <v>Finance</v>
     <v>5</v>
     <v>XNYS</v>
@@ -13420,14 +13434,14 @@
     <v>2025</v>
     <v>68.709999999999994</v>
     <v>-1.4</v>
-    <v>-4.6089999999999994E-3</v>
+    <v>-8.0289999999999997E-3</v>
     <v>-2.051E-2</v>
-    <v>-0.31</v>
+    <v>-0.54</v>
     <v>44608724560</v>
     <v>68.260000000000005</v>
     <v>Vylor Inc. is focused in the seed business, including its global growth platforms in licensing, gene editing, hybrid wheat, and biofuels. The Company is a global seed producer utilizing cutting-edge technology, including advanced genetics and proprietary traits that increase yield, sustainability, and crop heal.</v>
     <v>XNYS</v>
-    <v>46297.855263888283</v>
+    <v>46297.867572546093</v>
     <v>New York Stock Exchange</v>
     <v>71.36</v>
     <v>75</v>
@@ -13436,15 +13450,15 @@
     <v>USD</v>
     <v>Vylor</v>
     <v>Vylor</v>
-    <v>81.706000000000003</v>
+    <v>83.412800000000004</v>
     <v>66.86</v>
-    <v>66.95</v>
+    <v>66.72</v>
     <v>Food &amp; Tobacco</v>
     <v>7100 NW 62nd Avenue, JOHNSTON, IA, 50131 US</v>
     <v>VYLR</v>
     <v>Acciones</v>
     <v>Vylor (XNYS:VYLR)</v>
-    <v>13479015</v>
+    <v>13484119</v>
   </rv>
   <rv s="2">
     <v>207</v>
@@ -13472,15 +13486,15 @@
     <v>275.17500000000001</v>
     <v>1.9172</v>
     <v>7.95</v>
-    <v>-6.8409999999999999E-4</v>
+    <v>-7.2009999999999997E-5</v>
     <v>2.9446E-2</v>
-    <v>-0.19</v>
+    <v>-0.02</v>
     <v>74335636674</v>
     <v>269.99</v>
     <v>Royal Caribbean Cruises Ltd. Es una compañía de cruceros, que posee y opera tres marcas de cruceros globales: Royal Caribbean International, Celebrity Cruises y Silversea Cruises. También tiene interés en TUI Cruises GmbH, que opera las marcas alemanas TUI Cruises y Hapag-Lloyd Cruises. Sus barcos ofrecen una selección de itinerarios mundiales que hacen escala en aproximadamente 1.000 destinos en los siete continentes. Royal Caribbean International ofrece cruceros y destinos terrestres que generalmente ofrecen un ambiente informal, así como una variedad de actividades y lugares de entretenimiento. Celebrity Cruises ofrece una amplia gama de itinerarios a destinos, incluyendo Alaska, Asia, Australia, Bermudas, Canadá, el Caribe, Europa, las Islas Galápagos, Hawái, nueva Zelanda, el Canal de Panamá y América del Sur, con cruceros de tres a 14 noches. También ofrece una variedad de destinos privados de tierra a través de Perfect Day at CocoCay, incluye parque acuático completo, tirolesa y otros.</v>
     <v>107950</v>
     <v>XNYS</v>
-    <v>46297.854797534375</v>
+    <v>46297.870494421091</v>
     <v>New York Stock Exchange</v>
     <v>209</v>
     <v>279.5</v>
@@ -13492,44 +13506,44 @@
     <v>ROYAL CARIBBEAN CRUISES LTD.</v>
     <v>17.144300000000001</v>
     <v>277.94</v>
-    <v>277.55</v>
+    <v>277.72000000000003</v>
     <v>Hotels &amp; Entertainment Services</v>
     <v>1050 Caribbean Way, MIAMI, FL, 33132 US</v>
     <v>RCL</v>
     <v>Acciones</v>
     <v>ROYAL CARIBBEAN CRUISES LTD. (XNYS:RCL)</v>
-    <v>3389481</v>
+    <v>3390259</v>
     <v>2973012</v>
   </rv>
   <rv s="2">
     <v>210</v>
   </rv>
-  <rv s="17">
+  <rv s="16">
     <v>es-ES</v>
     <v>av8wim</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
+    <v>58</v>
+    <v>59</v>
+    <v>EUR/JPY</v>
+    <v>60</v>
     <v>61</v>
+    <v>Finance</v>
     <v>62</v>
-    <v>EUR/JPY</v>
-    <v>63</v>
-    <v>64</v>
-    <v>Finance</v>
-    <v>65</v>
     <v>177.65</v>
-    <v>-0.06</v>
-    <v>-3.3770000000000002E-4</v>
+    <v>-0.1</v>
+    <v>-5.6280000000000002E-4</v>
     <v>177.69</v>
     <v>EUR</v>
-    <v>46297.855717592596</v>
+    <v>46297.872418981482</v>
     <v>177.89</v>
     <v>187.93</v>
     <v>176.61</v>
     <v>172.2</v>
     <v>JPY</v>
     <v>Euro/Japanese Yen FX Cross Rate</v>
-    <v>177.63</v>
+    <v>177.59</v>
     <v>EURJPY</v>
     <v>Par de divisa</v>
     <v>EUR/JPY</v>
@@ -13537,32 +13551,32 @@
   <rv s="2">
     <v>212</v>
   </rv>
-  <rv s="17">
+  <rv s="16">
     <v>es-ES</v>
     <v>avv7r7</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>61</v>
+    <v>58</v>
+    <v>59</v>
+    <v>CHF/USD</v>
+    <v>60</v>
+    <v>63</v>
+    <v>Finance</v>
     <v>62</v>
-    <v>CHF/USD</v>
-    <v>63</v>
-    <v>66</v>
-    <v>Finance</v>
-    <v>65</v>
     <v>1.2024999999999999</v>
-    <v>4.1000000000000003E-3</v>
-    <v>3.4089999999999997E-3</v>
+    <v>3.5999999999999999E-3</v>
+    <v>2.993E-3</v>
     <v>1.2028000000000001</v>
     <v>CHF</v>
-    <v>46297.855671296296</v>
+    <v>46297.872430555559</v>
     <v>1.2152000000000001</v>
     <v>1.3149</v>
     <v>1.2011000000000001</v>
     <v>1.1926000000000001</v>
     <v>USD</v>
     <v>Swiss Franc/US Dollar FX Cross Rate</v>
-    <v>1.2069000000000001</v>
+    <v>1.2063999999999999</v>
     <v>CHFUSD</v>
     <v>Par de divisa</v>
     <v>CHF/USD</v>
@@ -13570,32 +13584,32 @@
   <rv s="2">
     <v>214</v>
   </rv>
-  <rv s="17">
+  <rv s="16">
     <v>es-ES</v>
     <v>avyosm</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>61</v>
+    <v>58</v>
+    <v>59</v>
+    <v>USD/KZT</v>
+    <v>60</v>
+    <v>64</v>
+    <v>Finance</v>
     <v>62</v>
-    <v>USD/KZT</v>
-    <v>63</v>
-    <v>67</v>
-    <v>Finance</v>
-    <v>65</v>
     <v>443.43</v>
-    <v>4.6900000000000004</v>
-    <v>1.0577000000000001E-2</v>
+    <v>4.6500000000000004</v>
+    <v>1.0486000000000001E-2</v>
     <v>443.43</v>
     <v>USD</v>
-    <v>46297.855717592596</v>
+    <v>46297.872430555559</v>
     <v>450.25</v>
     <v>549.66</v>
     <v>441.69</v>
     <v>439.14</v>
     <v>KZT</v>
     <v>US Dollar/Kazakhstan Tenge FX Spot Rate</v>
-    <v>448.12</v>
+    <v>448.08</v>
     <v>USDKZT</v>
     <v>Par de divisa</v>
     <v>USD/KZT</v>
@@ -13603,32 +13617,32 @@
   <rv s="2">
     <v>216</v>
   </rv>
-  <rv s="17">
+  <rv s="16">
     <v>es-ES</v>
     <v>av3wnm</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>61</v>
+    <v>58</v>
+    <v>59</v>
+    <v>CAD/USD</v>
+    <v>60</v>
+    <v>63</v>
+    <v>Finance</v>
     <v>62</v>
-    <v>CAD/USD</v>
-    <v>63</v>
-    <v>66</v>
-    <v>Finance</v>
-    <v>65</v>
     <v>0.70320000000000005</v>
-    <v>-1.1999999999999999E-3</v>
-    <v>-1.707E-3</v>
+    <v>-1.4E-3</v>
+    <v>-1.9910000000000001E-3</v>
     <v>0.70299999999999996</v>
     <v>CAD</v>
-    <v>46297.85565972222</v>
+    <v>46297.872418981482</v>
     <v>0.70379999999999998</v>
     <v>0.74170000000000003</v>
     <v>0.70120000000000005</v>
     <v>0.70099999999999996</v>
     <v>USD</v>
     <v>Canadian Dollar/US Dollar FX Cross Rate</v>
-    <v>0.70179999999999998</v>
+    <v>0.7016</v>
     <v>CADUSD</v>
     <v>Par de divisa</v>
     <v>CAD/USD</v>
@@ -13636,32 +13650,32 @@
   <rv s="2">
     <v>218</v>
   </rv>
-  <rv s="17">
+  <rv s="16">
     <v>es-ES</v>
     <v>avyn9c</v>
     <v>268435456</v>
     <v>1</v>
     <v>Con tecnología de Refinitiv</v>
-    <v>61</v>
+    <v>58</v>
+    <v>59</v>
+    <v>USD/EUR</v>
+    <v>60</v>
+    <v>65</v>
+    <v>Finance</v>
     <v>62</v>
-    <v>USD/EUR</v>
-    <v>63</v>
-    <v>68</v>
-    <v>Finance</v>
-    <v>65</v>
     <v>0.88959999999999995</v>
-    <v>-1.1000000000000001E-3</v>
-    <v>-1.237E-3</v>
+    <v>-5.9999999999999995E-4</v>
+    <v>-6.7460000000000003E-4</v>
     <v>0.88939999999999997</v>
     <v>USD</v>
-    <v>46297.85565972222</v>
+    <v>46297.872407407405</v>
     <v>0.8911</v>
     <v>0.89159999999999995</v>
     <v>0.8861</v>
     <v>0.82779999999999998</v>
     <v>EUR</v>
     <v>US Dollar/Euro FX Cross Rate</v>
-    <v>0.88829999999999998</v>
+    <v>0.88880000000000003</v>
     <v>USDEUR</v>
     <v>Par de divisa</v>
     <v>USD/EUR</v>
@@ -13673,7 +13687,7 @@
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="18">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="17">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -13872,53 +13886,6 @@
     <k n="Nombre" t="s"/>
     <k n="Nombre oficial" t="s"/>
     <k n="P/I"/>
-    <k n="Precio"/>
-    <k n="Precio (horario ampliado)"/>
-    <k n="Sector" t="s"/>
-    <k n="Sede central" t="s"/>
-    <k n="Símbolo bursátil" t="s"/>
-    <k n="Tipo de instrumento" t="s"/>
-    <k n="UniqueName" t="s"/>
-    <k n="Volumen"/>
-    <k n="Volumen promedio"/>
-  </s>
-  <s t="_linkedentitycore">
-    <k n="%EntityCulture" t="s"/>
-    <k n="%EntityId" t="s"/>
-    <k n="%EntityServiceId"/>
-    <k n="%IsRefreshable" t="b"/>
-    <k n="%ProviderInfo" t="s"/>
-    <k n="_CanonicalPropertyNames" t="spb"/>
-    <k n="_Display" t="spb"/>
-    <k n="_DisplayString" t="s"/>
-    <k n="_Flags" t="spb"/>
-    <k n="_Format" t="spb"/>
-    <k n="_Icon" t="s"/>
-    <k n="_SubLabel" t="spb"/>
-    <k n="Abreviatura de intercambio" t="s"/>
-    <k n="Acciones en circulación"/>
-    <k n="Año de constitución"/>
-    <k n="Apertura"/>
-    <k n="Beta"/>
-    <k n="Cambio"/>
-    <k n="Cambio % (horario ampliado)"/>
-    <k n="Cambio (%)"/>
-    <k n="Cambio (horario ampliado)"/>
-    <k n="Capitalización de mercado"/>
-    <k n="Cierre anterior"/>
-    <k n="Descripción" t="s"/>
-    <k n="Empleados"/>
-    <k n="ExchangeID" t="s"/>
-    <k n="Hora de la última operación"/>
-    <k n="Intercambio" t="s"/>
-    <k n="LearnMoreOnLink" t="r"/>
-    <k n="Máximo"/>
-    <k n="Máximo en 52 semanas"/>
-    <k n="Mínimo"/>
-    <k n="Mínimo en 52 semanas"/>
-    <k n="Moneda" t="s"/>
-    <k n="Nombre" t="s"/>
-    <k n="Nombre oficial" t="s"/>
     <k n="Precio"/>
     <k n="Precio (horario ampliado)"/>
     <k n="Sector" t="s"/>
@@ -14317,7 +14284,7 @@
 
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
-  <spbArrays count="14">
+  <spbArrays count="13">
     <a count="46">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
@@ -14504,53 +14471,6 @@
       <v t="s">_Flags</v>
       <v t="s">UniqueName</v>
       <v t="s">_DisplayString</v>
-      <v t="s">ExchangeID</v>
-      <v t="s">%ProviderInfo</v>
-    </a>
-    <a count="45">
-      <v t="s">%EntityServiceId</v>
-      <v t="s">_Format</v>
-      <v t="s">%IsRefreshable</v>
-      <v t="s">_CanonicalPropertyNames</v>
-      <v t="s">%EntityCulture</v>
-      <v t="s">%EntityId</v>
-      <v t="s">_Icon</v>
-      <v t="s">_Display</v>
-      <v t="s">Nombre</v>
-      <v t="s">_SubLabel</v>
-      <v t="s">Precio</v>
-      <v t="s">Precio (horario ampliado)</v>
-      <v t="s">Intercambio</v>
-      <v t="s">Nombre oficial</v>
-      <v t="s">Hora de la última operación</v>
-      <v t="s">Símbolo bursátil</v>
-      <v t="s">Abreviatura de intercambio</v>
-      <v t="s">Cambio</v>
-      <v t="s">Cambio (horario ampliado)</v>
-      <v t="s">Cambio (%)</v>
-      <v t="s">Cambio % (horario ampliado)</v>
-      <v t="s">Moneda</v>
-      <v t="s">Cierre anterior</v>
-      <v t="s">Apertura</v>
-      <v t="s">Máximo</v>
-      <v t="s">Mínimo</v>
-      <v t="s">Máximo en 52 semanas</v>
-      <v t="s">Mínimo en 52 semanas</v>
-      <v t="s">Volumen</v>
-      <v t="s">Volumen promedio</v>
-      <v t="s">Capitalización de mercado</v>
-      <v t="s">Beta</v>
-      <v t="s">Acciones en circulación</v>
-      <v t="s">Descripción</v>
-      <v t="s">Empleados</v>
-      <v t="s">Sede central</v>
-      <v t="s">Sector</v>
-      <v t="s">Tipo de instrumento</v>
-      <v t="s">Año de constitución</v>
-      <v t="s">_Flags</v>
-      <v t="s">UniqueName</v>
-      <v t="s">_DisplayString</v>
-      <v t="s">LearnMoreOnLink</v>
       <v t="s">ExchangeID</v>
       <v t="s">%ProviderInfo</v>
     </a>
@@ -14938,7 +14858,7 @@
       <v t="s">%ProviderInfo</v>
     </a>
   </spbArrays>
-  <spbData count="69">
+  <spbData count="66">
     <spb s="0">
       <v>P/E</v>
       <v>Beta</v>
@@ -15461,71 +15381,6 @@
       <v>%ProviderInfo</v>
       <v>Official name</v>
       <v>Previous close</v>
-      <v>LearnMoreOnLink</v>
-      <v>Ticker symbol</v>
-      <v>Volume average</v>
-      <v>Year incorporated</v>
-      <v>Instrument type</v>
-      <v>52 week high</v>
-      <v>52 week low</v>
-      <v>Shares outstanding</v>
-      <v>Change (Extended hours)</v>
-      <v>Market cap</v>
-      <v>Price (Extended hours)</v>
-      <v>Exchange abbreviation</v>
-      <v>Change % (Extended hours)</v>
-      <v>Last trade time</v>
-    </spb>
-    <spb s="1">
-      <v>4</v>
-      <v>Name</v>
-      <v>LearnMoreOnLink</v>
-    </spb>
-    <spb s="20">
-      <v>1</v>
-      <v>2</v>
-      <v>2</v>
-      <v>2</v>
-      <v>3</v>
-      <v>2</v>
-      <v>4</v>
-      <v>2</v>
-      <v>4</v>
-      <v>5</v>
-      <v>2</v>
-      <v>4</v>
-      <v>6</v>
-      <v>7</v>
-      <v>2</v>
-      <v>2</v>
-      <v>4</v>
-      <v>2</v>
-      <v>8</v>
-      <v>2</v>
-      <v>5</v>
-      <v>9</v>
-    </spb>
-    <spb s="21">
-      <v>Beta</v>
-      <v>Change</v>
-      <v>Currency</v>
-      <v>High</v>
-      <v>Low</v>
-      <v>Name</v>
-      <v>Price</v>
-      <v>Industry</v>
-      <v>Volume</v>
-      <v>Open</v>
-      <v>Employees</v>
-      <v>Change (%)</v>
-      <v>ExchangeID</v>
-      <v>UniqueName</v>
-      <v>Description</v>
-      <v>Exchange</v>
-      <v>Headquarters</v>
-      <v>%ProviderInfo</v>
-      <v>Official name</v>
-      <v>Previous close</v>
       <v>Ticker symbol</v>
       <v>Volume average</v>
       <v>Year incorporated</v>
@@ -15536,10 +15391,10 @@
       <v>Last trade time</v>
     </spb>
     <spb s="16">
-      <v>5</v>
+      <v>4</v>
       <v>Name</v>
     </spb>
-    <spb s="22">
+    <spb s="20">
       <v>1</v>
       <v>21</v>
       <v>21</v>
@@ -15558,7 +15413,7 @@
       <v>22</v>
       <v>9</v>
     </spb>
-    <spb s="23">
+    <spb s="21">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15592,11 +15447,11 @@
       <v>Last trade time</v>
     </spb>
     <spb s="1">
-      <v>6</v>
+      <v>5</v>
       <v>Name</v>
       <v>LearnMoreOnLink</v>
     </spb>
-    <spb s="24">
+    <spb s="22">
       <v>1</v>
       <v>1</v>
       <v>11</v>
@@ -15658,7 +15513,7 @@
       <v xml:space="preserve">desde el cierre </v>
       <v>GMT</v>
     </spb>
-    <spb s="25">
+    <spb s="23">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15694,11 +15549,11 @@
       <v>Last trade time</v>
     </spb>
     <spb s="1">
-      <v>7</v>
+      <v>6</v>
       <v>Name</v>
       <v>LearnMoreOnLink</v>
     </spb>
-    <spb s="26">
+    <spb s="24">
       <v>1</v>
       <v>1</v>
       <v>17</v>
@@ -15721,7 +15576,7 @@
       <v>5</v>
       <v>9</v>
     </spb>
-    <spb s="27">
+    <spb s="25">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15754,11 +15609,11 @@
       <v>Last trade time</v>
     </spb>
     <spb s="1">
-      <v>8</v>
+      <v>7</v>
       <v>Name</v>
       <v>LearnMoreOnLink</v>
     </spb>
-    <spb s="28">
+    <spb s="26">
       <v>1</v>
       <v>1</v>
       <v>11</v>
@@ -15778,7 +15633,7 @@
       <v>12</v>
       <v>24</v>
     </spb>
-    <spb s="29">
+    <spb s="27">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15812,7 +15667,7 @@
       <v>Last trade time</v>
     </spb>
     <spb s="16">
-      <v>9</v>
+      <v>8</v>
       <v>Name</v>
     </spb>
     <spb s="4">
@@ -15840,7 +15695,7 @@
       <v>5</v>
       <v>9</v>
     </spb>
-    <spb s="30">
+    <spb s="28">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15876,11 +15731,11 @@
       <v>Last trade time</v>
     </spb>
     <spb s="1">
-      <v>10</v>
+      <v>9</v>
       <v>Name</v>
       <v>LearnMoreOnLink</v>
     </spb>
-    <spb s="31">
+    <spb s="29">
       <v>1</v>
       <v>1</v>
       <v>15</v>
@@ -15903,7 +15758,7 @@
       <v>5</v>
       <v>9</v>
     </spb>
-    <spb s="32">
+    <spb s="30">
       <v>P/E</v>
       <v>Beta</v>
       <v>Change</v>
@@ -15938,10 +15793,10 @@
       <v>Last trade time</v>
     </spb>
     <spb s="16">
-      <v>11</v>
+      <v>10</v>
       <v>Name</v>
     </spb>
-    <spb s="33">
+    <spb s="31">
       <v>P/E</v>
       <v>Change</v>
       <v>Currency</v>
@@ -15975,10 +15830,10 @@
       <v>Last trade time</v>
     </spb>
     <spb s="16">
-      <v>12</v>
+      <v>11</v>
       <v>Name</v>
     </spb>
-    <spb s="34">
+    <spb s="32">
       <v>1</v>
       <v>2</v>
       <v>2</v>
@@ -16000,7 +15855,7 @@
       <v>5</v>
       <v>9</v>
     </spb>
-    <spb s="35">
+    <spb s="33">
       <v>Change</v>
       <v>Currency</v>
       <v>High</v>
@@ -16020,14 +15875,14 @@
       <v>Last trade time</v>
     </spb>
     <spb s="16">
-      <v>13</v>
+      <v>12</v>
       <v>Name</v>
     </spb>
-    <spb s="36">
+    <spb s="34">
       <v>2</v>
       <v>2</v>
     </spb>
-    <spb s="37">
+    <spb s="35">
       <v>25</v>
       <v>25</v>
       <v>25</v>
@@ -16041,10 +15896,10 @@
       <v>25</v>
       <v>9</v>
     </spb>
-    <spb s="38">
+    <spb s="36">
       <v>GMT</v>
     </spb>
-    <spb s="37">
+    <spb s="35">
       <v>2</v>
       <v>2</v>
       <v>2</v>
@@ -16058,7 +15913,7 @@
       <v>2</v>
       <v>9</v>
     </spb>
-    <spb s="37">
+    <spb s="35">
       <v>26</v>
       <v>26</v>
       <v>26</v>
@@ -16072,7 +15927,7 @@
       <v>26</v>
       <v>9</v>
     </spb>
-    <spb s="37">
+    <spb s="35">
       <v>11</v>
       <v>11</v>
       <v>11</v>
@@ -16091,7 +15946,7 @@
 </file>
 
 <file path=xl/richData/rdsupportingpropertybagstructure.xml><?xml version="1.0" encoding="utf-8"?>
-<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="39">
+<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="37">
   <s>
     <k n="P/I" t="s"/>
     <k n="Beta" t="s"/>
@@ -16380,66 +16235,6 @@
     <k n="Precio (horario ampliado)" t="s"/>
     <k n="Cambio % (horario ampliado)" t="s"/>
     <k n="Hora de la última operación" t="s"/>
-  </s>
-  <s>
-    <k n="Beta" t="s"/>
-    <k n="Cambio" t="s"/>
-    <k n="Moneda" t="s"/>
-    <k n="Máximo" t="s"/>
-    <k n="Mínimo" t="s"/>
-    <k n="Nombre" t="s"/>
-    <k n="Precio" t="s"/>
-    <k n="Sector" t="s"/>
-    <k n="Volumen" t="s"/>
-    <k n="Apertura" t="s"/>
-    <k n="Empleados" t="s"/>
-    <k n="Cambio (%)" t="s"/>
-    <k n="ExchangeID" t="s"/>
-    <k n="UniqueName" t="s"/>
-    <k n="Descripción" t="s"/>
-    <k n="Intercambio" t="s"/>
-    <k n="Sede central" t="s"/>
-    <k n="%ProviderInfo" t="s"/>
-    <k n="Nombre oficial" t="s"/>
-    <k n="Cierre anterior" t="s"/>
-    <k n="LearnMoreOnLink" t="s"/>
-    <k n="Símbolo bursátil" t="s"/>
-    <k n="Volumen promedio" t="s"/>
-    <k n="Año de constitución" t="s"/>
-    <k n="Tipo de instrumento" t="s"/>
-    <k n="Máximo en 52 semanas" t="s"/>
-    <k n="Mínimo en 52 semanas" t="s"/>
-    <k n="Acciones en circulación" t="s"/>
-    <k n="Cambio (horario ampliado)" t="s"/>
-    <k n="Capitalización de mercado" t="s"/>
-    <k n="Precio (horario ampliado)" t="s"/>
-    <k n="Abreviatura de intercambio" t="s"/>
-    <k n="Cambio % (horario ampliado)" t="s"/>
-    <k n="Hora de la última operación" t="s"/>
-  </s>
-  <s>
-    <k n="Beta" t="i"/>
-    <k n="Cambio" t="i"/>
-    <k n="Máximo" t="i"/>
-    <k n="Mínimo" t="i"/>
-    <k n="Nombre" t="i"/>
-    <k n="Precio" t="i"/>
-    <k n="Volumen" t="i"/>
-    <k n="Apertura" t="i"/>
-    <k n="Empleados" t="i"/>
-    <k n="Cambio (%)" t="i"/>
-    <k n="Cierre anterior" t="i"/>
-    <k n="Volumen promedio" t="i"/>
-    <k n="`%EntityServiceId" t="i"/>
-    <k n="Año de constitución" t="i"/>
-    <k n="Máximo en 52 semanas" t="i"/>
-    <k n="Mínimo en 52 semanas" t="i"/>
-    <k n="Acciones en circulación" t="i"/>
-    <k n="Cambio (horario ampliado)" t="i"/>
-    <k n="Capitalización de mercado" t="i"/>
-    <k n="Precio (horario ampliado)" t="i"/>
-    <k n="Cambio % (horario ampliado)" t="i"/>
-    <k n="Hora de la última operación" t="i"/>
   </s>
   <s>
     <k n="Beta" t="s"/>
@@ -19674,7 +19469,7 @@
       </c>
       <c r="AR12" s="19">
         <f ca="1">I12*'Framework Notes'!E4-AP12+AQ12</f>
-        <v>8184418.1247199997</v>
+        <v>8182131.9509599991</v>
       </c>
       <c r="AS12" s="103">
         <v>262620</v>
@@ -19690,15 +19485,15 @@
       </c>
       <c r="AW12" s="20">
         <f t="shared" ca="1" si="9"/>
-        <v>31.164489089635214</v>
+        <v>31.155783835808389</v>
       </c>
       <c r="AX12" s="20">
         <f t="shared" ca="1" si="10"/>
-        <v>17.730541864644714</v>
+        <v>17.725589148526861</v>
       </c>
       <c r="AY12" s="20">
         <f t="shared" ca="1" si="11"/>
-        <v>3.6238275407980778</v>
+        <v>3.6228152880870983</v>
       </c>
       <c r="AZ12" s="21">
         <v>1600000</v>
@@ -19737,19 +19532,19 @@
       </c>
       <c r="BJ12" s="25">
         <f ca="1">((BD12*BH12+$AP12-$AQ12)/$H12)/'Framework Notes'!E4</f>
-        <v>25.834476944290799</v>
+        <v>25.840295847820116</v>
       </c>
       <c r="BK12" s="25">
         <f ca="1">((BF12*BI12+$AP12-$AQ12)/$H12)/'Framework Notes'!E4</f>
-        <v>56.218865232300772</v>
+        <v>56.231527851869963</v>
       </c>
       <c r="BL12" s="23">
         <f t="shared" ca="1" si="18"/>
-        <v>-0.10264695553418879</v>
+        <v>-0.1026065355912541</v>
       </c>
       <c r="BM12" s="23">
         <f t="shared" ca="1" si="19"/>
-        <v>4.8334361539594806E-2</v>
+        <v>4.8381582213031127E-2</v>
       </c>
       <c r="BN12" s="95" t="s">
         <v>655</v>
@@ -23701,7 +23496,7 @@
       </c>
       <c r="G29" s="12">
         <f t="array" aca="1" ref="G29" ca="1">_FV(A29,"Precio")</f>
-        <v>90.26</v>
+        <v>90.29</v>
       </c>
       <c r="H29" s="13">
         <f t="array" aca="1" ref="H29" ca="1">_FV(A29,"Acciones en circulación",TRUE())/1000000</f>
@@ -23709,7 +23504,7 @@
       </c>
       <c r="I29" s="14">
         <f t="shared" ca="1" si="25"/>
-        <v>81020.589256000007</v>
+        <v>81047.518324000004</v>
       </c>
       <c r="J29" s="91">
         <v>0</v>
@@ -23822,7 +23617,7 @@
       </c>
       <c r="AR29" s="19">
         <f t="shared" ca="1" si="21"/>
-        <v>116104.58925600001</v>
+        <v>116131.518324</v>
       </c>
       <c r="AS29" s="103">
         <v>5000</v>
@@ -23838,15 +23633,15 @@
       </c>
       <c r="AW29" s="20">
         <f t="shared" ca="1" si="9"/>
-        <v>23.220917851200003</v>
+        <v>23.2263036648</v>
       </c>
       <c r="AX29" s="20">
         <f t="shared" ca="1" si="10"/>
-        <v>17.195584901658769</v>
+        <v>17.19957321149289</v>
       </c>
       <c r="AY29" s="20">
         <f t="shared" ca="1" si="11"/>
-        <v>4.4944291896411572</v>
+        <v>4.4954716186273371</v>
       </c>
       <c r="AZ29" s="21">
         <v>34500</v>
@@ -23893,11 +23688,11 @@
       </c>
       <c r="BL29" s="23">
         <f t="shared" ca="1" si="18"/>
-        <v>-2.8510406550612655E-2</v>
+        <v>-2.8574973085230049E-2</v>
       </c>
       <c r="BM29" s="23">
         <f t="shared" ca="1" si="19"/>
-        <v>0.27776808429597666</v>
+        <v>0.27768316207158628</v>
       </c>
       <c r="BN29" s="95" t="s">
         <v>813</v>
@@ -24789,7 +24584,7 @@
       </c>
       <c r="AR33" s="19">
         <f ca="1">I33*'Framework Notes'!E5-AP33+AQ33</f>
-        <v>184071.95246321603</v>
+        <v>183997.057296896</v>
       </c>
       <c r="AS33" s="103">
         <v>4159</v>
@@ -24805,15 +24600,15 @@
       </c>
       <c r="AW33" s="20">
         <f t="shared" ca="1" si="9"/>
-        <v>44.258704607649925</v>
+        <v>44.240696633059869</v>
       </c>
       <c r="AX33" s="20">
         <f t="shared" ca="1" si="10"/>
-        <v>25.74432901583441</v>
+        <v>25.733854167398043</v>
       </c>
       <c r="AY33" s="20">
         <f t="shared" ca="1" si="11"/>
-        <v>5.1488658031668821</v>
+        <v>5.1467708334796081</v>
       </c>
       <c r="AZ33" s="21">
         <v>27296</v>
@@ -24852,19 +24647,19 @@
       </c>
       <c r="BJ33" s="25">
         <f ca="1">((BD33*BH33+$AP33-$AQ33)/$H33)/'Framework Notes'!E5</f>
-        <v>30.700094497149948</v>
+        <v>30.712818342680933</v>
       </c>
       <c r="BK33" s="25">
         <f ca="1">((BF33*BI33+$AP33-$AQ33)/$H33)/'Framework Notes'!E5</f>
-        <v>81.783038619456818</v>
+        <v>81.816934109600837</v>
       </c>
       <c r="BL33" s="23">
         <f t="shared" ca="1" si="18"/>
-        <v>-0.17871128323244889</v>
+        <v>-0.17864321687010432</v>
       </c>
       <c r="BM33" s="23">
         <f t="shared" ca="1" si="19"/>
-        <v>-9.1931624013175117E-4</v>
+        <v>-8.3651492258784987E-4</v>
       </c>
       <c r="BN33" s="95" t="s">
         <v>655</v>
@@ -24912,7 +24707,7 @@
       </c>
       <c r="G34" s="12">
         <f t="array" aca="1" ref="G34" ca="1">_FV(A34,"Precio")</f>
-        <v>281.02999999999997</v>
+        <v>281.16000000000003</v>
       </c>
       <c r="H34" s="13">
         <f t="array" aca="1" ref="H34" ca="1">_FV(A34,"Acciones en circulación",TRUE())/1000000</f>
@@ -24920,7 +24715,7 @@
       </c>
       <c r="I34" s="14">
         <f t="shared" ca="1" si="25"/>
-        <v>54197.338074999992</v>
+        <v>54222.408900000002</v>
       </c>
       <c r="J34" s="90">
         <v>0</v>
@@ -25033,7 +24828,7 @@
       </c>
       <c r="AR34" s="19">
         <f ca="1">I34-AP34+AQ34</f>
-        <v>51754.338074999992</v>
+        <v>51779.408900000002</v>
       </c>
       <c r="AS34" s="103">
         <v>1427.3</v>
@@ -25049,15 +24844,15 @@
       </c>
       <c r="AW34" s="20">
         <f t="shared" ca="1" si="9"/>
-        <v>36.260308326910945</v>
+        <v>36.277873537448329</v>
       </c>
       <c r="AX34" s="20">
         <f t="shared" ca="1" si="10"/>
-        <v>22.404475357142854</v>
+        <v>22.415328528138531</v>
       </c>
       <c r="AY34" s="20">
         <f t="shared" ca="1" si="11"/>
-        <v>6.7476320827900906</v>
+        <v>6.7509007692307694</v>
       </c>
       <c r="AZ34" s="21">
         <v>9341</v>
@@ -25104,11 +24899,11 @@
       </c>
       <c r="BL34" s="23">
         <f t="shared" ca="1" si="18"/>
-        <v>-9.0612575439264487E-2</v>
+        <v>-9.0696685722298609E-2</v>
       </c>
       <c r="BM34" s="23">
         <f t="shared" ca="1" si="19"/>
-        <v>5.4929233984469361E-2</v>
+        <v>5.4831662373014289E-2</v>
       </c>
       <c r="BN34" s="95" t="s">
         <v>655</v>
@@ -25520,7 +25315,7 @@
       </c>
       <c r="AR36" s="19">
         <f ca="1">I36*'Framework Notes'!E6-AP36+AQ36</f>
-        <v>7179590.2402809989</v>
+        <v>7178877.9676539991</v>
       </c>
       <c r="AS36" s="103">
         <v>1054825</v>
@@ -25536,15 +25331,15 @@
       </c>
       <c r="AW36" s="20">
         <f t="shared" ref="AW36:AW66" ca="1" si="35">AR36/AS36</f>
-        <v>6.8064278342672946</v>
+        <v>6.8057525823278731</v>
       </c>
       <c r="AX36" s="20">
         <f t="shared" ref="AX36:AX66" ca="1" si="36">AR36/AU36</f>
-        <v>4.4703348585730716</v>
+        <v>4.4698913656930159</v>
       </c>
       <c r="AY36" s="20">
         <f t="shared" ref="AY36:AY66" ca="1" si="37">AR36/AV36</f>
-        <v>1.6135709149336643</v>
+        <v>1.6134108358266448</v>
       </c>
       <c r="AZ36" s="21">
         <v>2601577</v>
@@ -25583,19 +25378,19 @@
       </c>
       <c r="BJ36" s="25">
         <f ca="1">((BD36*BH36+$AP36-$AQ36)/$H36)/'Framework Notes'!E6</f>
-        <v>84.461727254840383</v>
+        <v>84.469267134081122</v>
       </c>
       <c r="BK36" s="25">
         <f ca="1">((BF36*BI36+$AP36-$AQ36)/$H36)/'Framework Notes'!E6</f>
-        <v>499.59074351036043</v>
+        <v>499.63534186275382</v>
       </c>
       <c r="BL36" s="23">
         <f t="shared" ref="BL36:BL71" ca="1" si="43">IF($BJ36&lt;=0,-0.99,MAX(-0.99,($BJ36/G36)^(1/5)-1))</f>
-        <v>-2.1276014339567495E-2</v>
+        <v>-2.1258540869841691E-2</v>
       </c>
       <c r="BM36" s="23">
         <f t="shared" ref="BM36:BM71" ca="1" si="44">IF(BK36&lt;=0,-0.99,MAX(-0.99,(BK36/G36)^(1/5)-1))</f>
-        <v>0.39653272387404837</v>
+        <v>0.39655765661568876</v>
       </c>
       <c r="BN36" s="96" t="s">
         <v>881</v>
@@ -26740,7 +26535,7 @@
       </c>
       <c r="AR41" s="19">
         <f ca="1">I41*'Framework Notes'!E8-AP41+AQ41</f>
-        <v>79812.988599450298</v>
+        <v>79861.582536520815</v>
       </c>
       <c r="AS41" s="103">
         <v>2993</v>
@@ -26756,15 +26551,15 @@
       </c>
       <c r="AW41" s="20">
         <f t="shared" ca="1" si="35"/>
-        <v>26.666551486618875</v>
+        <v>26.682787349322023</v>
       </c>
       <c r="AX41" s="20">
         <f t="shared" ca="1" si="36"/>
-        <v>29.022904945254655</v>
+        <v>29.04057546782575</v>
       </c>
       <c r="AY41" s="20">
         <f t="shared" ca="1" si="37"/>
-        <v>4.4063925688428363</v>
+        <v>4.4090753898592618</v>
       </c>
       <c r="AZ41" s="21">
         <v>8834</v>
@@ -26803,19 +26598,19 @@
       </c>
       <c r="BJ41" s="25">
         <f ca="1">((BD41*BH41+$AP41-$AQ41)/$H41)/'Framework Notes'!E8</f>
-        <v>377.75057357137786</v>
+        <v>377.53806762314912</v>
       </c>
       <c r="BK41" s="25">
         <f ca="1">((BF41*BI41+$AP41-$AQ41)/$H41)/'Framework Notes'!E8</f>
-        <v>695.80053908178468</v>
+        <v>695.4091121358565</v>
       </c>
       <c r="BL41" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-4.3917367129005291E-2</v>
+        <v>-4.4024961396064599E-2</v>
       </c>
       <c r="BM41" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>8.0317360170602203E-2</v>
+        <v>8.0195784952558524E-2</v>
       </c>
       <c r="BN41" s="95" t="s">
         <v>655</v>
@@ -28683,7 +28478,7 @@
       </c>
       <c r="AR49" s="19">
         <f ca="1">I49*'Framework Notes'!E7-AP49+AQ49</f>
-        <v>6504.3786754399989</v>
+        <v>6502.5823292799996</v>
       </c>
       <c r="AS49" s="103">
         <v>209</v>
@@ -28699,15 +28494,15 @@
       </c>
       <c r="AW49" s="20">
         <f t="shared" ca="1" si="35"/>
-        <v>31.121429069090905</v>
+        <v>31.112834111387556</v>
       </c>
       <c r="AX49" s="20">
         <f t="shared" ca="1" si="36"/>
-        <v>17.252993834058351</v>
+        <v>17.248228990132624</v>
       </c>
       <c r="AY49" s="20">
         <f t="shared" ca="1" si="37"/>
-        <v>13.301387884335377</v>
+        <v>13.297714374805725</v>
       </c>
       <c r="AZ49" s="21">
         <v>2539</v>
@@ -28746,19 +28541,19 @@
       </c>
       <c r="BJ49" s="25">
         <f ca="1">((BD49*BH49+$AP49-$AQ49)/$H49)/'Framework Notes'!E7</f>
-        <v>20.348211110931992</v>
+        <v>20.354011627212188</v>
       </c>
       <c r="BK49" s="25">
         <f ca="1">((BF49*BI49+$AP49-$AQ49)/$H49)/'Framework Notes'!E7</f>
-        <v>47.56354574859364</v>
+        <v>47.577104342022544</v>
       </c>
       <c r="BL49" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-0.14136626193268187</v>
+        <v>-0.14131731462087893</v>
       </c>
       <c r="BM49" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>1.7554189459976222E-2</v>
+        <v>1.7612196197866581E-2</v>
       </c>
       <c r="BN49" s="95" t="s">
         <v>813</v>
@@ -29269,7 +29064,7 @@
         <v>1469</v>
       </c>
       <c r="BT51" s="96" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
     </row>
     <row r="52" spans="1:72" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29540,7 +29335,7 @@
       </c>
       <c r="G53" s="12">
         <f t="array" aca="1" ref="G53" ca="1">_FV(A53,"Precio")</f>
-        <v>223.37</v>
+        <v>223.33</v>
       </c>
       <c r="H53" s="13">
         <f t="array" aca="1" ref="H53" ca="1">_FV(A53,"Acciones en circulación",TRUE())/1000000</f>
@@ -29548,7 +29343,7 @@
       </c>
       <c r="I53" s="14">
         <f t="shared" ca="1" si="25"/>
-        <v>43211.529599000001</v>
+        <v>43203.791491000004</v>
       </c>
       <c r="J53" s="91">
         <v>0</v>
@@ -29661,7 +29456,7 @@
       </c>
       <c r="AR53" s="19">
         <f t="shared" ca="1" si="48"/>
-        <v>49661.529599000001</v>
+        <v>49653.791491000004</v>
       </c>
       <c r="AS53" s="103">
         <v>1160</v>
@@ -29677,15 +29472,15 @@
       </c>
       <c r="AW53" s="20">
         <f t="shared" ca="1" si="35"/>
-        <v>42.811663447413792</v>
+        <v>42.804992664655174</v>
       </c>
       <c r="AX53" s="20">
         <f t="shared" ca="1" si="36"/>
-        <v>16.171126538261152</v>
+        <v>16.168606802670141</v>
       </c>
       <c r="AY53" s="20">
         <f t="shared" ca="1" si="37"/>
-        <v>1.5792638045856389</v>
+        <v>1.5790177285187306</v>
       </c>
       <c r="AZ53" s="21">
         <v>12926</v>
@@ -29732,11 +29527,11 @@
       </c>
       <c r="BL53" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-0.10402565468210778</v>
+        <v>-0.10399356189879871</v>
       </c>
       <c r="BM53" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>8.9526465424403234E-2</v>
+        <v>8.9565491024797828E-2</v>
       </c>
       <c r="BN53" s="95" t="s">
         <v>655</v>
@@ -32092,7 +31887,7 @@
       </c>
       <c r="AR63" s="19">
         <f ca="1">I63*'Framework Notes'!E7-AP63+AQ63</f>
-        <v>3252.0104122585999</v>
+        <v>3251.2277646632001</v>
       </c>
       <c r="AS63" s="103">
         <v>50.7</v>
@@ -32108,15 +31903,15 @@
       </c>
       <c r="AW63" s="20">
         <f t="shared" ca="1" si="35"/>
-        <v>64.142217204311635</v>
+        <v>64.126780368110445</v>
       </c>
       <c r="AX63" s="20">
         <f t="shared" ca="1" si="36"/>
-        <v>12.853796095883794</v>
+        <v>12.850702627127273</v>
       </c>
       <c r="AY63" s="20">
         <f t="shared" ca="1" si="37"/>
-        <v>4.5997318419499296</v>
+        <v>4.5986248439366335</v>
       </c>
       <c r="AZ63" s="21">
         <v>1833</v>
@@ -32155,19 +31950,19 @@
       </c>
       <c r="BJ63" s="25">
         <f ca="1">((BD63*BH63+$AP63-$AQ63)/$H63)/'Framework Notes'!$E$7</f>
-        <v>16.189112054319917</v>
+        <v>16.193726966536083</v>
       </c>
       <c r="BK63" s="25">
         <f ca="1">((BF63*BI63+$AP63-$AQ63)/$H63)/'Framework Notes'!$E$7</f>
-        <v>70.754156606861741</v>
+        <v>70.774325978756508</v>
       </c>
       <c r="BL63" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-0.14236121690776071</v>
+        <v>-0.14231232631440394</v>
       </c>
       <c r="BM63" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>0.15188785108403979</v>
+        <v>0.15195351565242254</v>
       </c>
       <c r="BN63" s="95" t="s">
         <v>655</v>
@@ -32580,7 +32375,7 @@
       </c>
       <c r="AR65" s="19">
         <f ca="1">I65*'Framework Notes'!$E$7-AP65+AQ65</f>
-        <v>45379.19832798234</v>
+        <v>45366.563047752083</v>
       </c>
       <c r="AS65" s="103">
         <v>2771</v>
@@ -32596,15 +32391,15 @@
       </c>
       <c r="AW65" s="20">
         <f t="shared" ca="1" si="35"/>
-        <v>16.376469984836643</v>
+        <v>16.371910157976213</v>
       </c>
       <c r="AX65" s="20">
         <f t="shared" ca="1" si="36"/>
-        <v>13.237805813297065</v>
+        <v>13.234119908912509</v>
       </c>
       <c r="AY65" s="20">
         <f t="shared" ca="1" si="37"/>
-        <v>3.5898424434761758</v>
+        <v>3.5888428959538077</v>
       </c>
       <c r="AZ65" s="21">
         <v>5000</v>
@@ -32643,19 +32438,19 @@
       </c>
       <c r="BJ65" s="25">
         <f ca="1">((BD65*BH65+$AP65-$AQ65)/$H65)/'Framework Notes'!$E$7</f>
-        <v>2497.0051950740412</v>
+        <v>2497.7169981513143</v>
       </c>
       <c r="BK65" s="25">
         <f ca="1">((BF65*BI65+$AP65-$AQ65)/$H65)/'Framework Notes'!$E$7</f>
-        <v>7824.3485654585529</v>
+        <v>7826.5789954943157</v>
       </c>
       <c r="BL65" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-3.4826531129340421E-2</v>
+        <v>-3.4771510409060902E-2</v>
       </c>
       <c r="BM65" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>0.21286125877407347</v>
+        <v>0.21293039919515744</v>
       </c>
       <c r="BN65" s="95" t="s">
         <v>655</v>
@@ -33923,7 +33718,7 @@
       </c>
       <c r="G71" s="12">
         <f t="shared" ca="1" si="63"/>
-        <v>83.84</v>
+        <v>83.72</v>
       </c>
       <c r="H71" s="13">
         <f t="shared" ca="1" si="64"/>
@@ -33931,7 +33726,7 @@
       </c>
       <c r="I71" s="14">
         <f t="shared" ca="1" si="65"/>
-        <v>1251.1191680000002</v>
+        <v>1249.328444</v>
       </c>
       <c r="J71" s="90">
         <v>2</v>
@@ -34044,7 +33839,7 @@
       </c>
       <c r="AR71" s="19">
         <f t="shared" ca="1" si="51"/>
-        <v>1612.019168</v>
+        <v>1610.2284439999999</v>
       </c>
       <c r="AS71" s="103">
         <v>54.2</v>
@@ -34060,15 +33855,15 @@
       </c>
       <c r="AW71" s="20">
         <f t="shared" ca="1" si="56"/>
-        <v>29.742051070110701</v>
+        <v>29.709011881918816</v>
       </c>
       <c r="AX71" s="20">
         <f t="shared" ca="1" si="57"/>
-        <v>16.791866333333335</v>
+        <v>16.773212958333332</v>
       </c>
       <c r="AY71" s="20">
         <f t="shared" ca="1" si="58"/>
-        <v>2.0042511102822331</v>
+        <v>2.0020246723859256</v>
       </c>
       <c r="AZ71" s="21">
         <v>1127.5999999999999</v>
@@ -34115,11 +33910,11 @@
       </c>
       <c r="BL71" s="23">
         <f t="shared" ca="1" si="43"/>
-        <v>-0.12639805699229911</v>
+        <v>-0.12614776511385184</v>
       </c>
       <c r="BM71" s="23">
         <f t="shared" ca="1" si="44"/>
-        <v>0.10119407329009977</v>
+        <v>0.10150957159610163</v>
       </c>
       <c r="BN71" s="96" t="s">
         <v>519</v>
@@ -34425,10 +34220,10 @@
         <v>1</v>
       </c>
       <c r="K73" s="90">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L73" s="90">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M73" s="90">
         <v>0</v>
@@ -34447,20 +34242,20 @@
       </c>
       <c r="R73" s="15">
         <f t="shared" ref="R73" si="81">SUM(J73:N73)+SUM(P73:Q73)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S73" s="16">
         <f t="shared" ref="S73" si="82">ROUND(R73/16*10,2)</f>
-        <v>4.38</v>
+        <v>5.63</v>
       </c>
       <c r="T73" s="90">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="U73" s="90">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V73" s="90">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W73" s="90">
         <v>9</v>
@@ -34475,15 +34270,15 @@
         <v>5</v>
       </c>
       <c r="AA73" s="90">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="AB73" s="15">
         <f t="shared" ref="AB73" si="83">SUM(T73:AA73)</f>
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="AC73" s="16">
         <f t="shared" si="53"/>
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="AD73" s="90">
         <v>14</v>
@@ -34498,28 +34293,28 @@
         <v>9</v>
       </c>
       <c r="AH73" s="90">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI73" s="90">
         <v>6</v>
       </c>
       <c r="AJ73" s="90">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AK73" s="90">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="AL73" s="15">
         <f t="shared" ref="AL73" si="84">SUM(AD73:AK73)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AM73" s="16">
         <f t="shared" si="55"/>
-        <v>6.43</v>
+        <v>6.57</v>
       </c>
       <c r="AN73" s="17">
         <f t="shared" ref="AN73" si="85">ROUND(S73*0.2+AC73*0.4+AM73*0.4,2)</f>
-        <v>5.81</v>
+        <v>6.31</v>
       </c>
       <c r="AO73" s="18" t="s">
         <v>78</v>
@@ -34574,18 +34369,18 @@
         <v>6.9649967314435138E-2</v>
       </c>
       <c r="BD73" s="98">
-        <v>2046</v>
+        <v>2200</v>
       </c>
       <c r="BE73" s="23">
         <f t="shared" si="70"/>
-        <v>0.11354441696879736</v>
+        <v>0.12982441421042812</v>
       </c>
       <c r="BF73">
-        <v>3295</v>
+        <v>3320</v>
       </c>
       <c r="BG73" s="23">
         <f t="shared" si="71"/>
-        <v>0.22489116666880382</v>
+        <v>0.22674426314293461</v>
       </c>
       <c r="BH73" s="24">
         <v>14</v>
@@ -34595,19 +34390,19 @@
       </c>
       <c r="BJ73" s="25">
         <f t="shared" ca="1" si="72"/>
-        <v>36.098837523006729</v>
+        <v>39.330271764219205</v>
       </c>
       <c r="BK73" s="25">
         <f t="shared" ca="1" si="73"/>
-        <v>101.81565836725639</v>
+        <v>102.64000383695345</v>
       </c>
       <c r="BL73" s="23">
         <f t="shared" ref="BL73" ca="1" si="92">IF($BJ73&lt;=0,-0.99,MAX(-0.99,($BJ73/G73)^(1/5)-1))</f>
-        <v>-0.11597332684733153</v>
+        <v>-0.10068442478381578</v>
       </c>
       <c r="BM73" s="23">
         <f t="shared" ref="BM73" ca="1" si="93">IF(BK73&lt;=0,-0.99,MAX(-0.99,(BK73/G73)^(1/5)-1))</f>
-        <v>8.7751373438704316E-2</v>
+        <v>8.9507081704458091E-2</v>
       </c>
       <c r="BN73" s="96" t="s">
         <v>813</v>
@@ -34628,7 +34423,7 @@
         <v>1228</v>
       </c>
       <c r="BT73" s="96" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
     </row>
     <row r="74" spans="1:72" x14ac:dyDescent="0.25">
@@ -34925,7 +34720,7 @@
       </c>
       <c r="E4" s="29">
         <f t="array" aca="1" ref="E4" ca="1">_FV(D4,"Precio")</f>
-        <v>177.63</v>
+        <v>177.59</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34937,7 +34732,7 @@
       </c>
       <c r="E5" s="30">
         <f t="array" aca="1" ref="E5" ca="1">_FV(D5,"Precio")</f>
-        <v>1.2069000000000001</v>
+        <v>1.2063999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34949,7 +34744,7 @@
       </c>
       <c r="E6" s="31">
         <f t="array" aca="1" ref="E6" ca="1">_FV(D6,"Precio")</f>
-        <v>448.12</v>
+        <v>448.08</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34958,7 +34753,7 @@
       </c>
       <c r="E7" s="30">
         <f t="array" aca="1" ref="E7" ca="1">_FV(D7,"Precio")</f>
-        <v>0.70179999999999998</v>
+        <v>0.7016</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34970,7 +34765,7 @@
       </c>
       <c r="E8" s="87">
         <f t="array" aca="1" ref="E8" ca="1">_FV(D8,"Precio")</f>
-        <v>0.88829999999999998</v>
+        <v>0.88880000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -36754,7 +36549,7 @@
       </c>
       <c r="J16" s="50">
         <f ca="1">'Watchlist Ratings'!AW12</f>
-        <v>31.164489089635214</v>
+        <v>31.155783835808389</v>
       </c>
       <c r="L16" t="s">
         <v>255</v>
@@ -36773,7 +36568,7 @@
       </c>
       <c r="Q16" s="23">
         <f ca="1">'Watchlist Ratings'!BM12</f>
-        <v>4.8334361539594806E-2</v>
+        <v>4.8381582213031127E-2</v>
       </c>
       <c r="S16" t="str">
         <f ca="1">'Watchlist Ratings'!B12</f>
@@ -36801,7 +36596,7 @@
       </c>
       <c r="Z16">
         <f ca="1">'Watchlist Ratings'!AW12</f>
-        <v>31.164489089635214</v>
+        <v>31.155783835808389</v>
       </c>
       <c r="AA16" t="str">
         <f ca="1">'Watchlist Ratings'!B12</f>
@@ -36809,11 +36604,11 @@
       </c>
       <c r="AB16">
         <f ca="1">'Watchlist Ratings'!BL12</f>
-        <v>-0.10264695553418879</v>
+        <v>-0.1026065355912541</v>
       </c>
       <c r="AC16">
         <f ca="1">'Watchlist Ratings'!BM12</f>
-        <v>4.8334361539594806E-2</v>
+        <v>4.8381582213031127E-2</v>
       </c>
       <c r="AE16" t="s">
         <v>232</v>
@@ -39099,7 +38894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E261"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -43528,6 +43323,23 @@
         <v>858</v>
       </c>
     </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>914</v>
+      </c>
+      <c r="B261" s="183">
+        <v>46297</v>
+      </c>
+      <c r="C261" t="s">
+        <v>915</v>
+      </c>
+      <c r="D261" t="s">
+        <v>916</v>
+      </c>
+      <c r="E261" t="s">
+        <v>917</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>